<commit_message>
Agrega columna "Nuevo" al Excel del catálogo
Columna K con menú desplegable sí/no para marcar mercadería recién llegada
(alimenta la sección ✨ Novedades vía convertir.py). Incluye ejemplos y una
línea en la hoja Instrucciones.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Kialo_Catalogo.xlsx
+++ b/tools/Kialo_Catalogo.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17540" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Productos" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,14 +12,14 @@
     <sheet name="Instrucciones" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,29 +29,38 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="003B4756"/>
+      <color rgb="FF3B4756"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="003B4756"/>
+      <color rgb="FF3B4756"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
   <fills count="23">
@@ -64,107 +72,107 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003B4756"/>
+        <fgColor rgb="FF3B4756"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002B2B2B"/>
+        <fgColor rgb="FF2B2B2B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="009AA0A6"/>
+        <fgColor rgb="FF9AA0A6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0655A"/>
+        <fgColor rgb="FFF0655A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F7A8C4"/>
+        <fgColor rgb="FFF7A8C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E85A9B"/>
+        <fgColor rgb="FFE85A9B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4C040"/>
+        <fgColor rgb="FFF4C040"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F29B50"/>
+        <fgColor rgb="FFF29B50"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="006CB94E"/>
+        <fgColor rgb="FF6CB94E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003FB6A8"/>
+        <fgColor rgb="FF3FB6A8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007CC1EC"/>
+        <fgColor rgb="FF7CC1EC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003E8FD0"/>
+        <fgColor rgb="FF3E8FD0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002C3E7A"/>
+        <fgColor rgb="FF2C3E7A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="009B6FC9"/>
+        <fgColor rgb="FF9B6FC9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B79BE0"/>
+        <fgColor rgb="FFB79BE0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D8C4A3"/>
+        <fgColor rgb="FFD8C4A3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EFE6D3"/>
+        <fgColor rgb="FFEFE6D3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="009C6B4A"/>
+        <fgColor rgb="FF9C6B4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D4AF37"/>
+        <fgColor rgb="FFD4AF37"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007D2240"/>
+        <fgColor rgb="FF7D2240"/>
       </patternFill>
     </fill>
   </fills>
@@ -178,23 +186,24 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D2C5"/>
+        <color rgb="FFD9D2C5"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D2C5"/>
+        <color rgb="FFD9D2C5"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D2C5"/>
+        <color rgb="FFD9D2C5"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D2C5"/>
+        <color rgb="FFD9D2C5"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -232,9 +241,15 @@
     <xf numFmtId="0" fontId="0" fillId="22" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -597,19 +612,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J200"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K200"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="3" max="4"/>
+    <col width="30" customWidth="1" min="5" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="8" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -663,8 +676,13 @@
           <t>Colores (por nombre, separados por coma)</t>
         </is>
       </c>
-    </row>
-    <row r="2">
+      <c r="K1" s="29" t="inlineStr">
+        <is>
+          <t>Nuevo (sí / no)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Boina con lazo</t>
@@ -711,8 +729,13 @@
           <t>blanco, rojo, rosa, negro, beige, lila</t>
         </is>
       </c>
-    </row>
-    <row r="3">
+      <c r="K2" s="30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Pantys panda</t>
@@ -752,9 +775,14 @@
           <t>Algodón con elastano</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="30" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Lentes de sol niña</t>
@@ -796,7 +824,12 @@
           <t>Marco flexible · UV400</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="30" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n"/>
@@ -809,6 +842,7 @@
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
+      <c r="K5" s="30" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n"/>
@@ -821,6 +855,7 @@
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
+      <c r="K6" s="30" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n"/>
@@ -833,6 +868,7 @@
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
+      <c r="K7" s="30" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
@@ -845,6 +881,7 @@
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
+      <c r="K8" s="30" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n"/>
@@ -857,6 +894,7 @@
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
+      <c r="K9" s="30" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
@@ -869,6 +907,7 @@
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
+      <c r="K10" s="30" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>
@@ -881,6 +920,7 @@
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
+      <c r="K11" s="30" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
@@ -893,6 +933,7 @@
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
+      <c r="K12" s="30" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -905,6 +946,7 @@
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
+      <c r="K13" s="30" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -917,6 +959,7 @@
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
+      <c r="K14" s="30" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
@@ -929,6 +972,7 @@
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
+      <c r="K15" s="30" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
@@ -941,6 +985,7 @@
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
+      <c r="K16" s="30" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
@@ -953,6 +998,7 @@
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
+      <c r="K17" s="30" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
@@ -965,6 +1011,7 @@
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
+      <c r="K18" s="30" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
@@ -977,6 +1024,7 @@
       <c r="H19" s="3" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
+      <c r="K19" s="30" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
@@ -989,6 +1037,7 @@
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
+      <c r="K20" s="30" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
@@ -1001,6 +1050,7 @@
       <c r="H21" s="3" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
+      <c r="K21" s="30" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
@@ -1013,6 +1063,7 @@
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
+      <c r="K22" s="30" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
@@ -1025,6 +1076,7 @@
       <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
+      <c r="K23" s="30" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
@@ -1037,6 +1089,7 @@
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
+      <c r="K24" s="30" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
@@ -1049,6 +1102,7 @@
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
+      <c r="K25" s="30" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
@@ -1061,6 +1115,7 @@
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
+      <c r="K26" s="30" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
@@ -1073,6 +1128,7 @@
       <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
+      <c r="K27" s="30" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
@@ -1085,6 +1141,7 @@
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
+      <c r="K28" s="30" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
@@ -1097,6 +1154,7 @@
       <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
+      <c r="K29" s="30" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
@@ -1109,6 +1167,7 @@
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
+      <c r="K30" s="30" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
@@ -1121,6 +1180,7 @@
       <c r="H31" s="3" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
+      <c r="K31" s="30" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n"/>
@@ -1133,6 +1193,7 @@
       <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
+      <c r="K32" s="30" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n"/>
@@ -1145,6 +1206,7 @@
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
+      <c r="K33" s="30" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n"/>
@@ -1157,6 +1219,7 @@
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
+      <c r="K34" s="30" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>
@@ -1169,6 +1232,7 @@
       <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
+      <c r="K35" s="30" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
@@ -1181,6 +1245,7 @@
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
+      <c r="K36" s="30" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
@@ -1193,6 +1258,7 @@
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
+      <c r="K37" s="30" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
@@ -1205,6 +1271,7 @@
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
+      <c r="K38" s="30" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
@@ -1217,6 +1284,7 @@
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
+      <c r="K39" s="30" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
@@ -1229,6 +1297,7 @@
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
+      <c r="K40" s="30" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
@@ -1241,6 +1310,7 @@
       <c r="H41" s="3" t="n"/>
       <c r="I41" s="3" t="n"/>
       <c r="J41" s="3" t="n"/>
+      <c r="K41" s="30" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
@@ -1253,6 +1323,7 @@
       <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="n"/>
       <c r="J42" s="3" t="n"/>
+      <c r="K42" s="30" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
@@ -1265,6 +1336,7 @@
       <c r="H43" s="3" t="n"/>
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="3" t="n"/>
+      <c r="K43" s="30" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
@@ -1277,6 +1349,7 @@
       <c r="H44" s="3" t="n"/>
       <c r="I44" s="3" t="n"/>
       <c r="J44" s="3" t="n"/>
+      <c r="K44" s="30" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
@@ -1289,6 +1362,7 @@
       <c r="H45" s="3" t="n"/>
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="3" t="n"/>
+      <c r="K45" s="30" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
@@ -1301,6 +1375,7 @@
       <c r="H46" s="3" t="n"/>
       <c r="I46" s="3" t="n"/>
       <c r="J46" s="3" t="n"/>
+      <c r="K46" s="30" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
@@ -1313,6 +1388,7 @@
       <c r="H47" s="3" t="n"/>
       <c r="I47" s="3" t="n"/>
       <c r="J47" s="3" t="n"/>
+      <c r="K47" s="30" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -1325,6 +1401,7 @@
       <c r="H48" s="3" t="n"/>
       <c r="I48" s="3" t="n"/>
       <c r="J48" s="3" t="n"/>
+      <c r="K48" s="30" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
@@ -1337,6 +1414,7 @@
       <c r="H49" s="3" t="n"/>
       <c r="I49" s="3" t="n"/>
       <c r="J49" s="3" t="n"/>
+      <c r="K49" s="30" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
@@ -1349,6 +1427,7 @@
       <c r="H50" s="3" t="n"/>
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="3" t="n"/>
+      <c r="K50" s="30" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
@@ -1361,6 +1440,7 @@
       <c r="H51" s="3" t="n"/>
       <c r="I51" s="3" t="n"/>
       <c r="J51" s="3" t="n"/>
+      <c r="K51" s="30" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
@@ -1373,6 +1453,7 @@
       <c r="H52" s="3" t="n"/>
       <c r="I52" s="3" t="n"/>
       <c r="J52" s="3" t="n"/>
+      <c r="K52" s="30" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n"/>
@@ -1385,6 +1466,7 @@
       <c r="H53" s="3" t="n"/>
       <c r="I53" s="3" t="n"/>
       <c r="J53" s="3" t="n"/>
+      <c r="K53" s="30" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
@@ -1397,6 +1479,7 @@
       <c r="H54" s="3" t="n"/>
       <c r="I54" s="3" t="n"/>
       <c r="J54" s="3" t="n"/>
+      <c r="K54" s="30" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
@@ -1409,6 +1492,7 @@
       <c r="H55" s="3" t="n"/>
       <c r="I55" s="3" t="n"/>
       <c r="J55" s="3" t="n"/>
+      <c r="K55" s="30" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
@@ -1421,6 +1505,7 @@
       <c r="H56" s="3" t="n"/>
       <c r="I56" s="3" t="n"/>
       <c r="J56" s="3" t="n"/>
+      <c r="K56" s="30" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
@@ -1433,6 +1518,7 @@
       <c r="H57" s="3" t="n"/>
       <c r="I57" s="3" t="n"/>
       <c r="J57" s="3" t="n"/>
+      <c r="K57" s="30" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
@@ -1445,6 +1531,7 @@
       <c r="H58" s="3" t="n"/>
       <c r="I58" s="3" t="n"/>
       <c r="J58" s="3" t="n"/>
+      <c r="K58" s="30" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
@@ -1457,6 +1544,7 @@
       <c r="H59" s="3" t="n"/>
       <c r="I59" s="3" t="n"/>
       <c r="J59" s="3" t="n"/>
+      <c r="K59" s="30" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
@@ -1469,6 +1557,7 @@
       <c r="H60" s="3" t="n"/>
       <c r="I60" s="3" t="n"/>
       <c r="J60" s="3" t="n"/>
+      <c r="K60" s="30" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
@@ -1481,6 +1570,7 @@
       <c r="H61" s="3" t="n"/>
       <c r="I61" s="3" t="n"/>
       <c r="J61" s="3" t="n"/>
+      <c r="K61" s="30" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
@@ -1493,6 +1583,7 @@
       <c r="H62" s="3" t="n"/>
       <c r="I62" s="3" t="n"/>
       <c r="J62" s="3" t="n"/>
+      <c r="K62" s="30" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>
@@ -1505,6 +1596,7 @@
       <c r="H63" s="3" t="n"/>
       <c r="I63" s="3" t="n"/>
       <c r="J63" s="3" t="n"/>
+      <c r="K63" s="30" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>
@@ -1517,6 +1609,7 @@
       <c r="H64" s="3" t="n"/>
       <c r="I64" s="3" t="n"/>
       <c r="J64" s="3" t="n"/>
+      <c r="K64" s="30" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
@@ -1529,6 +1622,7 @@
       <c r="H65" s="3" t="n"/>
       <c r="I65" s="3" t="n"/>
       <c r="J65" s="3" t="n"/>
+      <c r="K65" s="30" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
@@ -1541,6 +1635,7 @@
       <c r="H66" s="3" t="n"/>
       <c r="I66" s="3" t="n"/>
       <c r="J66" s="3" t="n"/>
+      <c r="K66" s="30" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
@@ -1553,6 +1648,7 @@
       <c r="H67" s="3" t="n"/>
       <c r="I67" s="3" t="n"/>
       <c r="J67" s="3" t="n"/>
+      <c r="K67" s="30" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n"/>
@@ -1565,6 +1661,7 @@
       <c r="H68" s="3" t="n"/>
       <c r="I68" s="3" t="n"/>
       <c r="J68" s="3" t="n"/>
+      <c r="K68" s="30" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
@@ -1577,6 +1674,7 @@
       <c r="H69" s="3" t="n"/>
       <c r="I69" s="3" t="n"/>
       <c r="J69" s="3" t="n"/>
+      <c r="K69" s="30" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
@@ -1589,6 +1687,7 @@
       <c r="H70" s="3" t="n"/>
       <c r="I70" s="3" t="n"/>
       <c r="J70" s="3" t="n"/>
+      <c r="K70" s="30" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
@@ -1601,6 +1700,7 @@
       <c r="H71" s="3" t="n"/>
       <c r="I71" s="3" t="n"/>
       <c r="J71" s="3" t="n"/>
+      <c r="K71" s="30" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
@@ -1613,6 +1713,7 @@
       <c r="H72" s="3" t="n"/>
       <c r="I72" s="3" t="n"/>
       <c r="J72" s="3" t="n"/>
+      <c r="K72" s="30" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
@@ -1625,6 +1726,7 @@
       <c r="H73" s="3" t="n"/>
       <c r="I73" s="3" t="n"/>
       <c r="J73" s="3" t="n"/>
+      <c r="K73" s="30" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
@@ -1637,6 +1739,7 @@
       <c r="H74" s="3" t="n"/>
       <c r="I74" s="3" t="n"/>
       <c r="J74" s="3" t="n"/>
+      <c r="K74" s="30" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
@@ -1649,6 +1752,7 @@
       <c r="H75" s="3" t="n"/>
       <c r="I75" s="3" t="n"/>
       <c r="J75" s="3" t="n"/>
+      <c r="K75" s="30" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n"/>
@@ -1661,6 +1765,7 @@
       <c r="H76" s="3" t="n"/>
       <c r="I76" s="3" t="n"/>
       <c r="J76" s="3" t="n"/>
+      <c r="K76" s="30" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
@@ -1673,6 +1778,7 @@
       <c r="H77" s="3" t="n"/>
       <c r="I77" s="3" t="n"/>
       <c r="J77" s="3" t="n"/>
+      <c r="K77" s="30" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
@@ -1685,6 +1791,7 @@
       <c r="H78" s="3" t="n"/>
       <c r="I78" s="3" t="n"/>
       <c r="J78" s="3" t="n"/>
+      <c r="K78" s="30" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
@@ -1697,6 +1804,7 @@
       <c r="H79" s="3" t="n"/>
       <c r="I79" s="3" t="n"/>
       <c r="J79" s="3" t="n"/>
+      <c r="K79" s="30" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
@@ -1709,6 +1817,7 @@
       <c r="H80" s="3" t="n"/>
       <c r="I80" s="3" t="n"/>
       <c r="J80" s="3" t="n"/>
+      <c r="K80" s="30" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
@@ -1721,6 +1830,7 @@
       <c r="H81" s="3" t="n"/>
       <c r="I81" s="3" t="n"/>
       <c r="J81" s="3" t="n"/>
+      <c r="K81" s="30" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
@@ -1733,6 +1843,7 @@
       <c r="H82" s="3" t="n"/>
       <c r="I82" s="3" t="n"/>
       <c r="J82" s="3" t="n"/>
+      <c r="K82" s="30" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
@@ -1745,6 +1856,7 @@
       <c r="H83" s="3" t="n"/>
       <c r="I83" s="3" t="n"/>
       <c r="J83" s="3" t="n"/>
+      <c r="K83" s="30" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
@@ -1757,6 +1869,7 @@
       <c r="H84" s="3" t="n"/>
       <c r="I84" s="3" t="n"/>
       <c r="J84" s="3" t="n"/>
+      <c r="K84" s="30" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n"/>
@@ -1769,6 +1882,7 @@
       <c r="H85" s="3" t="n"/>
       <c r="I85" s="3" t="n"/>
       <c r="J85" s="3" t="n"/>
+      <c r="K85" s="30" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n"/>
@@ -1781,6 +1895,7 @@
       <c r="H86" s="3" t="n"/>
       <c r="I86" s="3" t="n"/>
       <c r="J86" s="3" t="n"/>
+      <c r="K86" s="30" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n"/>
@@ -1793,6 +1908,7 @@
       <c r="H87" s="3" t="n"/>
       <c r="I87" s="3" t="n"/>
       <c r="J87" s="3" t="n"/>
+      <c r="K87" s="30" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
@@ -1805,6 +1921,7 @@
       <c r="H88" s="3" t="n"/>
       <c r="I88" s="3" t="n"/>
       <c r="J88" s="3" t="n"/>
+      <c r="K88" s="30" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n"/>
@@ -1817,6 +1934,7 @@
       <c r="H89" s="3" t="n"/>
       <c r="I89" s="3" t="n"/>
       <c r="J89" s="3" t="n"/>
+      <c r="K89" s="30" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n"/>
@@ -1829,6 +1947,7 @@
       <c r="H90" s="3" t="n"/>
       <c r="I90" s="3" t="n"/>
       <c r="J90" s="3" t="n"/>
+      <c r="K90" s="30" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n"/>
@@ -1841,6 +1960,7 @@
       <c r="H91" s="3" t="n"/>
       <c r="I91" s="3" t="n"/>
       <c r="J91" s="3" t="n"/>
+      <c r="K91" s="30" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n"/>
@@ -1853,6 +1973,7 @@
       <c r="H92" s="3" t="n"/>
       <c r="I92" s="3" t="n"/>
       <c r="J92" s="3" t="n"/>
+      <c r="K92" s="30" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n"/>
@@ -1865,6 +1986,7 @@
       <c r="H93" s="3" t="n"/>
       <c r="I93" s="3" t="n"/>
       <c r="J93" s="3" t="n"/>
+      <c r="K93" s="30" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n"/>
@@ -1877,6 +1999,7 @@
       <c r="H94" s="3" t="n"/>
       <c r="I94" s="3" t="n"/>
       <c r="J94" s="3" t="n"/>
+      <c r="K94" s="30" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n"/>
@@ -1889,6 +2012,7 @@
       <c r="H95" s="3" t="n"/>
       <c r="I95" s="3" t="n"/>
       <c r="J95" s="3" t="n"/>
+      <c r="K95" s="30" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n"/>
@@ -1901,6 +2025,7 @@
       <c r="H96" s="3" t="n"/>
       <c r="I96" s="3" t="n"/>
       <c r="J96" s="3" t="n"/>
+      <c r="K96" s="30" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n"/>
@@ -1913,6 +2038,7 @@
       <c r="H97" s="3" t="n"/>
       <c r="I97" s="3" t="n"/>
       <c r="J97" s="3" t="n"/>
+      <c r="K97" s="30" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n"/>
@@ -1925,6 +2051,7 @@
       <c r="H98" s="3" t="n"/>
       <c r="I98" s="3" t="n"/>
       <c r="J98" s="3" t="n"/>
+      <c r="K98" s="30" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n"/>
@@ -1937,6 +2064,7 @@
       <c r="H99" s="3" t="n"/>
       <c r="I99" s="3" t="n"/>
       <c r="J99" s="3" t="n"/>
+      <c r="K99" s="30" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n"/>
@@ -1949,6 +2077,7 @@
       <c r="H100" s="3" t="n"/>
       <c r="I100" s="3" t="n"/>
       <c r="J100" s="3" t="n"/>
+      <c r="K100" s="30" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n"/>
@@ -1961,6 +2090,7 @@
       <c r="H101" s="3" t="n"/>
       <c r="I101" s="3" t="n"/>
       <c r="J101" s="3" t="n"/>
+      <c r="K101" s="30" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n"/>
@@ -1973,6 +2103,7 @@
       <c r="H102" s="3" t="n"/>
       <c r="I102" s="3" t="n"/>
       <c r="J102" s="3" t="n"/>
+      <c r="K102" s="30" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n"/>
@@ -1985,6 +2116,7 @@
       <c r="H103" s="3" t="n"/>
       <c r="I103" s="3" t="n"/>
       <c r="J103" s="3" t="n"/>
+      <c r="K103" s="30" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n"/>
@@ -1997,6 +2129,7 @@
       <c r="H104" s="3" t="n"/>
       <c r="I104" s="3" t="n"/>
       <c r="J104" s="3" t="n"/>
+      <c r="K104" s="30" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n"/>
@@ -2009,6 +2142,7 @@
       <c r="H105" s="3" t="n"/>
       <c r="I105" s="3" t="n"/>
       <c r="J105" s="3" t="n"/>
+      <c r="K105" s="30" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n"/>
@@ -2021,6 +2155,7 @@
       <c r="H106" s="3" t="n"/>
       <c r="I106" s="3" t="n"/>
       <c r="J106" s="3" t="n"/>
+      <c r="K106" s="30" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n"/>
@@ -2033,6 +2168,7 @@
       <c r="H107" s="3" t="n"/>
       <c r="I107" s="3" t="n"/>
       <c r="J107" s="3" t="n"/>
+      <c r="K107" s="30" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n"/>
@@ -2045,6 +2181,7 @@
       <c r="H108" s="3" t="n"/>
       <c r="I108" s="3" t="n"/>
       <c r="J108" s="3" t="n"/>
+      <c r="K108" s="30" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n"/>
@@ -2057,6 +2194,7 @@
       <c r="H109" s="3" t="n"/>
       <c r="I109" s="3" t="n"/>
       <c r="J109" s="3" t="n"/>
+      <c r="K109" s="30" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n"/>
@@ -2069,6 +2207,7 @@
       <c r="H110" s="3" t="n"/>
       <c r="I110" s="3" t="n"/>
       <c r="J110" s="3" t="n"/>
+      <c r="K110" s="30" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n"/>
@@ -2081,6 +2220,7 @@
       <c r="H111" s="3" t="n"/>
       <c r="I111" s="3" t="n"/>
       <c r="J111" s="3" t="n"/>
+      <c r="K111" s="30" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n"/>
@@ -2093,6 +2233,7 @@
       <c r="H112" s="3" t="n"/>
       <c r="I112" s="3" t="n"/>
       <c r="J112" s="3" t="n"/>
+      <c r="K112" s="30" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n"/>
@@ -2105,6 +2246,7 @@
       <c r="H113" s="3" t="n"/>
       <c r="I113" s="3" t="n"/>
       <c r="J113" s="3" t="n"/>
+      <c r="K113" s="30" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n"/>
@@ -2117,6 +2259,7 @@
       <c r="H114" s="3" t="n"/>
       <c r="I114" s="3" t="n"/>
       <c r="J114" s="3" t="n"/>
+      <c r="K114" s="30" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n"/>
@@ -2129,6 +2272,7 @@
       <c r="H115" s="3" t="n"/>
       <c r="I115" s="3" t="n"/>
       <c r="J115" s="3" t="n"/>
+      <c r="K115" s="30" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n"/>
@@ -2141,6 +2285,7 @@
       <c r="H116" s="3" t="n"/>
       <c r="I116" s="3" t="n"/>
       <c r="J116" s="3" t="n"/>
+      <c r="K116" s="30" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n"/>
@@ -2153,6 +2298,7 @@
       <c r="H117" s="3" t="n"/>
       <c r="I117" s="3" t="n"/>
       <c r="J117" s="3" t="n"/>
+      <c r="K117" s="30" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n"/>
@@ -2165,6 +2311,7 @@
       <c r="H118" s="3" t="n"/>
       <c r="I118" s="3" t="n"/>
       <c r="J118" s="3" t="n"/>
+      <c r="K118" s="30" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n"/>
@@ -2177,6 +2324,7 @@
       <c r="H119" s="3" t="n"/>
       <c r="I119" s="3" t="n"/>
       <c r="J119" s="3" t="n"/>
+      <c r="K119" s="30" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n"/>
@@ -2189,6 +2337,7 @@
       <c r="H120" s="3" t="n"/>
       <c r="I120" s="3" t="n"/>
       <c r="J120" s="3" t="n"/>
+      <c r="K120" s="30" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n"/>
@@ -2201,6 +2350,7 @@
       <c r="H121" s="3" t="n"/>
       <c r="I121" s="3" t="n"/>
       <c r="J121" s="3" t="n"/>
+      <c r="K121" s="30" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n"/>
@@ -2213,6 +2363,7 @@
       <c r="H122" s="3" t="n"/>
       <c r="I122" s="3" t="n"/>
       <c r="J122" s="3" t="n"/>
+      <c r="K122" s="30" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n"/>
@@ -2225,6 +2376,7 @@
       <c r="H123" s="3" t="n"/>
       <c r="I123" s="3" t="n"/>
       <c r="J123" s="3" t="n"/>
+      <c r="K123" s="30" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n"/>
@@ -2237,6 +2389,7 @@
       <c r="H124" s="3" t="n"/>
       <c r="I124" s="3" t="n"/>
       <c r="J124" s="3" t="n"/>
+      <c r="K124" s="30" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n"/>
@@ -2249,6 +2402,7 @@
       <c r="H125" s="3" t="n"/>
       <c r="I125" s="3" t="n"/>
       <c r="J125" s="3" t="n"/>
+      <c r="K125" s="30" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n"/>
@@ -2261,6 +2415,7 @@
       <c r="H126" s="3" t="n"/>
       <c r="I126" s="3" t="n"/>
       <c r="J126" s="3" t="n"/>
+      <c r="K126" s="30" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n"/>
@@ -2273,6 +2428,7 @@
       <c r="H127" s="3" t="n"/>
       <c r="I127" s="3" t="n"/>
       <c r="J127" s="3" t="n"/>
+      <c r="K127" s="30" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n"/>
@@ -2285,6 +2441,7 @@
       <c r="H128" s="3" t="n"/>
       <c r="I128" s="3" t="n"/>
       <c r="J128" s="3" t="n"/>
+      <c r="K128" s="30" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n"/>
@@ -2297,6 +2454,7 @@
       <c r="H129" s="3" t="n"/>
       <c r="I129" s="3" t="n"/>
       <c r="J129" s="3" t="n"/>
+      <c r="K129" s="30" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n"/>
@@ -2309,6 +2467,7 @@
       <c r="H130" s="3" t="n"/>
       <c r="I130" s="3" t="n"/>
       <c r="J130" s="3" t="n"/>
+      <c r="K130" s="30" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n"/>
@@ -2321,6 +2480,7 @@
       <c r="H131" s="3" t="n"/>
       <c r="I131" s="3" t="n"/>
       <c r="J131" s="3" t="n"/>
+      <c r="K131" s="30" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n"/>
@@ -2333,6 +2493,7 @@
       <c r="H132" s="3" t="n"/>
       <c r="I132" s="3" t="n"/>
       <c r="J132" s="3" t="n"/>
+      <c r="K132" s="30" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n"/>
@@ -2345,6 +2506,7 @@
       <c r="H133" s="3" t="n"/>
       <c r="I133" s="3" t="n"/>
       <c r="J133" s="3" t="n"/>
+      <c r="K133" s="30" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n"/>
@@ -2357,6 +2519,7 @@
       <c r="H134" s="3" t="n"/>
       <c r="I134" s="3" t="n"/>
       <c r="J134" s="3" t="n"/>
+      <c r="K134" s="30" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n"/>
@@ -2369,6 +2532,7 @@
       <c r="H135" s="3" t="n"/>
       <c r="I135" s="3" t="n"/>
       <c r="J135" s="3" t="n"/>
+      <c r="K135" s="30" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n"/>
@@ -2381,6 +2545,7 @@
       <c r="H136" s="3" t="n"/>
       <c r="I136" s="3" t="n"/>
       <c r="J136" s="3" t="n"/>
+      <c r="K136" s="30" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n"/>
@@ -2393,6 +2558,7 @@
       <c r="H137" s="3" t="n"/>
       <c r="I137" s="3" t="n"/>
       <c r="J137" s="3" t="n"/>
+      <c r="K137" s="30" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n"/>
@@ -2405,6 +2571,7 @@
       <c r="H138" s="3" t="n"/>
       <c r="I138" s="3" t="n"/>
       <c r="J138" s="3" t="n"/>
+      <c r="K138" s="30" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n"/>
@@ -2417,6 +2584,7 @@
       <c r="H139" s="3" t="n"/>
       <c r="I139" s="3" t="n"/>
       <c r="J139" s="3" t="n"/>
+      <c r="K139" s="30" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n"/>
@@ -2429,6 +2597,7 @@
       <c r="H140" s="3" t="n"/>
       <c r="I140" s="3" t="n"/>
       <c r="J140" s="3" t="n"/>
+      <c r="K140" s="30" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n"/>
@@ -2441,6 +2610,7 @@
       <c r="H141" s="3" t="n"/>
       <c r="I141" s="3" t="n"/>
       <c r="J141" s="3" t="n"/>
+      <c r="K141" s="30" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n"/>
@@ -2453,6 +2623,7 @@
       <c r="H142" s="3" t="n"/>
       <c r="I142" s="3" t="n"/>
       <c r="J142" s="3" t="n"/>
+      <c r="K142" s="30" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n"/>
@@ -2465,6 +2636,7 @@
       <c r="H143" s="3" t="n"/>
       <c r="I143" s="3" t="n"/>
       <c r="J143" s="3" t="n"/>
+      <c r="K143" s="30" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n"/>
@@ -2477,6 +2649,7 @@
       <c r="H144" s="3" t="n"/>
       <c r="I144" s="3" t="n"/>
       <c r="J144" s="3" t="n"/>
+      <c r="K144" s="30" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n"/>
@@ -2489,6 +2662,7 @@
       <c r="H145" s="3" t="n"/>
       <c r="I145" s="3" t="n"/>
       <c r="J145" s="3" t="n"/>
+      <c r="K145" s="30" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n"/>
@@ -2501,6 +2675,7 @@
       <c r="H146" s="3" t="n"/>
       <c r="I146" s="3" t="n"/>
       <c r="J146" s="3" t="n"/>
+      <c r="K146" s="30" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n"/>
@@ -2513,6 +2688,7 @@
       <c r="H147" s="3" t="n"/>
       <c r="I147" s="3" t="n"/>
       <c r="J147" s="3" t="n"/>
+      <c r="K147" s="30" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n"/>
@@ -2525,6 +2701,7 @@
       <c r="H148" s="3" t="n"/>
       <c r="I148" s="3" t="n"/>
       <c r="J148" s="3" t="n"/>
+      <c r="K148" s="30" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n"/>
@@ -2537,6 +2714,7 @@
       <c r="H149" s="3" t="n"/>
       <c r="I149" s="3" t="n"/>
       <c r="J149" s="3" t="n"/>
+      <c r="K149" s="30" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n"/>
@@ -2549,6 +2727,7 @@
       <c r="H150" s="3" t="n"/>
       <c r="I150" s="3" t="n"/>
       <c r="J150" s="3" t="n"/>
+      <c r="K150" s="30" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n"/>
@@ -2561,6 +2740,7 @@
       <c r="H151" s="3" t="n"/>
       <c r="I151" s="3" t="n"/>
       <c r="J151" s="3" t="n"/>
+      <c r="K151" s="30" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n"/>
@@ -2573,6 +2753,7 @@
       <c r="H152" s="3" t="n"/>
       <c r="I152" s="3" t="n"/>
       <c r="J152" s="3" t="n"/>
+      <c r="K152" s="30" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="n"/>
@@ -2585,6 +2766,7 @@
       <c r="H153" s="3" t="n"/>
       <c r="I153" s="3" t="n"/>
       <c r="J153" s="3" t="n"/>
+      <c r="K153" s="30" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n"/>
@@ -2597,6 +2779,7 @@
       <c r="H154" s="3" t="n"/>
       <c r="I154" s="3" t="n"/>
       <c r="J154" s="3" t="n"/>
+      <c r="K154" s="30" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n"/>
@@ -2609,6 +2792,7 @@
       <c r="H155" s="3" t="n"/>
       <c r="I155" s="3" t="n"/>
       <c r="J155" s="3" t="n"/>
+      <c r="K155" s="30" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n"/>
@@ -2621,6 +2805,7 @@
       <c r="H156" s="3" t="n"/>
       <c r="I156" s="3" t="n"/>
       <c r="J156" s="3" t="n"/>
+      <c r="K156" s="30" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n"/>
@@ -2633,6 +2818,7 @@
       <c r="H157" s="3" t="n"/>
       <c r="I157" s="3" t="n"/>
       <c r="J157" s="3" t="n"/>
+      <c r="K157" s="30" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n"/>
@@ -2645,6 +2831,7 @@
       <c r="H158" s="3" t="n"/>
       <c r="I158" s="3" t="n"/>
       <c r="J158" s="3" t="n"/>
+      <c r="K158" s="30" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n"/>
@@ -2657,6 +2844,7 @@
       <c r="H159" s="3" t="n"/>
       <c r="I159" s="3" t="n"/>
       <c r="J159" s="3" t="n"/>
+      <c r="K159" s="30" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n"/>
@@ -2669,6 +2857,7 @@
       <c r="H160" s="3" t="n"/>
       <c r="I160" s="3" t="n"/>
       <c r="J160" s="3" t="n"/>
+      <c r="K160" s="30" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="n"/>
@@ -2681,6 +2870,7 @@
       <c r="H161" s="3" t="n"/>
       <c r="I161" s="3" t="n"/>
       <c r="J161" s="3" t="n"/>
+      <c r="K161" s="30" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n"/>
@@ -2693,6 +2883,7 @@
       <c r="H162" s="3" t="n"/>
       <c r="I162" s="3" t="n"/>
       <c r="J162" s="3" t="n"/>
+      <c r="K162" s="30" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n"/>
@@ -2705,6 +2896,7 @@
       <c r="H163" s="3" t="n"/>
       <c r="I163" s="3" t="n"/>
       <c r="J163" s="3" t="n"/>
+      <c r="K163" s="30" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n"/>
@@ -2717,6 +2909,7 @@
       <c r="H164" s="3" t="n"/>
       <c r="I164" s="3" t="n"/>
       <c r="J164" s="3" t="n"/>
+      <c r="K164" s="30" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n"/>
@@ -2729,6 +2922,7 @@
       <c r="H165" s="3" t="n"/>
       <c r="I165" s="3" t="n"/>
       <c r="J165" s="3" t="n"/>
+      <c r="K165" s="30" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n"/>
@@ -2741,6 +2935,7 @@
       <c r="H166" s="3" t="n"/>
       <c r="I166" s="3" t="n"/>
       <c r="J166" s="3" t="n"/>
+      <c r="K166" s="30" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n"/>
@@ -2753,6 +2948,7 @@
       <c r="H167" s="3" t="n"/>
       <c r="I167" s="3" t="n"/>
       <c r="J167" s="3" t="n"/>
+      <c r="K167" s="30" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n"/>
@@ -2765,6 +2961,7 @@
       <c r="H168" s="3" t="n"/>
       <c r="I168" s="3" t="n"/>
       <c r="J168" s="3" t="n"/>
+      <c r="K168" s="30" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n"/>
@@ -2777,6 +2974,7 @@
       <c r="H169" s="3" t="n"/>
       <c r="I169" s="3" t="n"/>
       <c r="J169" s="3" t="n"/>
+      <c r="K169" s="30" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n"/>
@@ -2789,6 +2987,7 @@
       <c r="H170" s="3" t="n"/>
       <c r="I170" s="3" t="n"/>
       <c r="J170" s="3" t="n"/>
+      <c r="K170" s="30" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n"/>
@@ -2801,6 +3000,7 @@
       <c r="H171" s="3" t="n"/>
       <c r="I171" s="3" t="n"/>
       <c r="J171" s="3" t="n"/>
+      <c r="K171" s="30" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n"/>
@@ -2813,6 +3013,7 @@
       <c r="H172" s="3" t="n"/>
       <c r="I172" s="3" t="n"/>
       <c r="J172" s="3" t="n"/>
+      <c r="K172" s="30" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n"/>
@@ -2825,6 +3026,7 @@
       <c r="H173" s="3" t="n"/>
       <c r="I173" s="3" t="n"/>
       <c r="J173" s="3" t="n"/>
+      <c r="K173" s="30" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n"/>
@@ -2837,6 +3039,7 @@
       <c r="H174" s="3" t="n"/>
       <c r="I174" s="3" t="n"/>
       <c r="J174" s="3" t="n"/>
+      <c r="K174" s="30" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n"/>
@@ -2849,6 +3052,7 @@
       <c r="H175" s="3" t="n"/>
       <c r="I175" s="3" t="n"/>
       <c r="J175" s="3" t="n"/>
+      <c r="K175" s="30" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n"/>
@@ -2861,6 +3065,7 @@
       <c r="H176" s="3" t="n"/>
       <c r="I176" s="3" t="n"/>
       <c r="J176" s="3" t="n"/>
+      <c r="K176" s="30" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n"/>
@@ -2873,6 +3078,7 @@
       <c r="H177" s="3" t="n"/>
       <c r="I177" s="3" t="n"/>
       <c r="J177" s="3" t="n"/>
+      <c r="K177" s="30" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n"/>
@@ -2885,6 +3091,7 @@
       <c r="H178" s="3" t="n"/>
       <c r="I178" s="3" t="n"/>
       <c r="J178" s="3" t="n"/>
+      <c r="K178" s="30" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n"/>
@@ -2897,6 +3104,7 @@
       <c r="H179" s="3" t="n"/>
       <c r="I179" s="3" t="n"/>
       <c r="J179" s="3" t="n"/>
+      <c r="K179" s="30" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n"/>
@@ -2909,6 +3117,7 @@
       <c r="H180" s="3" t="n"/>
       <c r="I180" s="3" t="n"/>
       <c r="J180" s="3" t="n"/>
+      <c r="K180" s="30" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n"/>
@@ -2921,6 +3130,7 @@
       <c r="H181" s="3" t="n"/>
       <c r="I181" s="3" t="n"/>
       <c r="J181" s="3" t="n"/>
+      <c r="K181" s="30" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n"/>
@@ -2933,6 +3143,7 @@
       <c r="H182" s="3" t="n"/>
       <c r="I182" s="3" t="n"/>
       <c r="J182" s="3" t="n"/>
+      <c r="K182" s="30" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n"/>
@@ -2945,6 +3156,7 @@
       <c r="H183" s="3" t="n"/>
       <c r="I183" s="3" t="n"/>
       <c r="J183" s="3" t="n"/>
+      <c r="K183" s="30" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n"/>
@@ -2957,6 +3169,7 @@
       <c r="H184" s="3" t="n"/>
       <c r="I184" s="3" t="n"/>
       <c r="J184" s="3" t="n"/>
+      <c r="K184" s="30" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n"/>
@@ -2969,6 +3182,7 @@
       <c r="H185" s="3" t="n"/>
       <c r="I185" s="3" t="n"/>
       <c r="J185" s="3" t="n"/>
+      <c r="K185" s="30" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n"/>
@@ -2981,6 +3195,7 @@
       <c r="H186" s="3" t="n"/>
       <c r="I186" s="3" t="n"/>
       <c r="J186" s="3" t="n"/>
+      <c r="K186" s="30" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n"/>
@@ -2993,6 +3208,7 @@
       <c r="H187" s="3" t="n"/>
       <c r="I187" s="3" t="n"/>
       <c r="J187" s="3" t="n"/>
+      <c r="K187" s="30" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n"/>
@@ -3005,6 +3221,7 @@
       <c r="H188" s="3" t="n"/>
       <c r="I188" s="3" t="n"/>
       <c r="J188" s="3" t="n"/>
+      <c r="K188" s="30" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n"/>
@@ -3017,6 +3234,7 @@
       <c r="H189" s="3" t="n"/>
       <c r="I189" s="3" t="n"/>
       <c r="J189" s="3" t="n"/>
+      <c r="K189" s="30" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n"/>
@@ -3029,6 +3247,7 @@
       <c r="H190" s="3" t="n"/>
       <c r="I190" s="3" t="n"/>
       <c r="J190" s="3" t="n"/>
+      <c r="K190" s="30" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n"/>
@@ -3041,6 +3260,7 @@
       <c r="H191" s="3" t="n"/>
       <c r="I191" s="3" t="n"/>
       <c r="J191" s="3" t="n"/>
+      <c r="K191" s="30" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n"/>
@@ -3053,6 +3273,7 @@
       <c r="H192" s="3" t="n"/>
       <c r="I192" s="3" t="n"/>
       <c r="J192" s="3" t="n"/>
+      <c r="K192" s="30" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n"/>
@@ -3065,6 +3286,7 @@
       <c r="H193" s="3" t="n"/>
       <c r="I193" s="3" t="n"/>
       <c r="J193" s="3" t="n"/>
+      <c r="K193" s="30" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n"/>
@@ -3077,6 +3299,7 @@
       <c r="H194" s="3" t="n"/>
       <c r="I194" s="3" t="n"/>
       <c r="J194" s="3" t="n"/>
+      <c r="K194" s="30" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n"/>
@@ -3089,6 +3312,7 @@
       <c r="H195" s="3" t="n"/>
       <c r="I195" s="3" t="n"/>
       <c r="J195" s="3" t="n"/>
+      <c r="K195" s="30" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n"/>
@@ -3101,6 +3325,7 @@
       <c r="H196" s="3" t="n"/>
       <c r="I196" s="3" t="n"/>
       <c r="J196" s="3" t="n"/>
+      <c r="K196" s="30" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n"/>
@@ -3113,6 +3338,7 @@
       <c r="H197" s="3" t="n"/>
       <c r="I197" s="3" t="n"/>
       <c r="J197" s="3" t="n"/>
+      <c r="K197" s="30" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n"/>
@@ -3125,6 +3351,7 @@
       <c r="H198" s="3" t="n"/>
       <c r="I198" s="3" t="n"/>
       <c r="J198" s="3" t="n"/>
+      <c r="K198" s="30" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n"/>
@@ -3137,6 +3364,7 @@
       <c r="H199" s="3" t="n"/>
       <c r="I199" s="3" t="n"/>
       <c r="J199" s="3" t="n"/>
+      <c r="K199" s="30" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n"/>
@@ -3149,11 +3377,15 @@
       <c r="H200" s="3" t="n"/>
       <c r="I200" s="3" t="n"/>
       <c r="J200" s="3" t="n"/>
+      <c r="K200" s="30" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="B2:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Categoría inválida" error="Usa: accesorios, ropa, zapatillas o disfraces" type="list">
       <formula1>"accesorios,ropa,zapatillas,tematicas"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Novedad" prompt="Pon 'sí' si es mercadería recién llegada (sale en ✨ Novedades)." type="list">
+      <formula1>"sí,no"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3167,7 +3399,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -3217,7 +3449,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>https://www.tiktok.com/@kialo.bebe?is_from_webapp=1&amp;sender_device=pc</t>
         </is>
       </c>
     </row>
@@ -3245,13 +3477,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="16" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Escribe el color por su NOMBRE. Estos son los disponibles:</t>
@@ -3276,7 +3508,7 @@
           <t>blanco</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
+      <c r="B4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -3284,7 +3516,7 @@
           <t>negro</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr"/>
+      <c r="B5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -3292,7 +3524,7 @@
           <t>gris</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr"/>
+      <c r="B6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -3300,7 +3532,7 @@
           <t>rojo</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr"/>
+      <c r="B7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -3308,7 +3540,7 @@
           <t>rosa</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr"/>
+      <c r="B8" s="11" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -3316,7 +3548,7 @@
           <t>fucsia</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr"/>
+      <c r="B9" s="12" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -3324,7 +3556,7 @@
           <t>amarillo</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr"/>
+      <c r="B10" s="13" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -3332,7 +3564,7 @@
           <t>naranja</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr"/>
+      <c r="B11" s="14" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -3340,7 +3572,7 @@
           <t>verde</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr"/>
+      <c r="B12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -3348,7 +3580,7 @@
           <t>turquesa</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr"/>
+      <c r="B13" s="16" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -3356,7 +3588,7 @@
           <t>celeste</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr"/>
+      <c r="B14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -3364,7 +3596,7 @@
           <t>azul</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr"/>
+      <c r="B15" s="18" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -3372,7 +3604,7 @@
           <t>azul marino</t>
         </is>
       </c>
-      <c r="B16" s="19" t="inlineStr"/>
+      <c r="B16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -3380,7 +3612,7 @@
           <t>morado</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr"/>
+      <c r="B17" s="20" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -3388,7 +3620,7 @@
           <t>lila</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr"/>
+      <c r="B18" s="21" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -3396,7 +3628,7 @@
           <t>beige</t>
         </is>
       </c>
-      <c r="B19" s="22" t="inlineStr"/>
+      <c r="B19" s="22" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -3404,7 +3636,7 @@
           <t>crema</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr"/>
+      <c r="B20" s="23" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -3412,7 +3644,7 @@
           <t>marrón</t>
         </is>
       </c>
-      <c r="B21" s="24" t="inlineStr"/>
+      <c r="B21" s="24" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -3420,7 +3652,7 @@
           <t>dorado</t>
         </is>
       </c>
-      <c r="B22" s="25" t="inlineStr"/>
+      <c r="B22" s="25" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -3428,7 +3660,7 @@
           <t>vino</t>
         </is>
       </c>
-      <c r="B23" s="26" t="inlineStr"/>
+      <c r="B23" s="26" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3449,12 +3681,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="27" t="inlineStr">
         <is>
           <t>📋 Cómo llenar esta plantilla — Kialo bebé</t>
@@ -3469,7 +3701,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr"/>
+      <c r="A4" s="28" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="28" t="inlineStr">
@@ -3528,7 +3760,11 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="inlineStr"/>
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Nuevo: escribe 'sí' si es mercadería recién llegada (aparece en la sección ✨ Novedades). Vacío o 'no' = normal.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="inlineStr">
@@ -3538,7 +3774,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr"/>
+      <c r="A15" s="28" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
@@ -3548,7 +3784,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="inlineStr"/>
+      <c r="A17" s="28" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Quita la columna Fotos del Excel (las fotos van por carpetas)
Las fotos ya no se escriben en el Excel: se arrastran a la carpeta de cada
producto y convertir.py las engancha por código. Reubica el menú "Nuevo"
(K->J) y actualiza la hoja Instrucciones al nuevo flujo.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/Kialo_Catalogo.xlsx
+++ b/tools/Kialo_Catalogo.xlsx
@@ -612,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K200"/>
+  <dimension ref="A1:J200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -621,7 +621,7 @@
     <col width="30" customWidth="1" min="5" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -648,35 +648,30 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Fotos (archivos, separados por coma)</t>
+          <t>Descripción corta</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Descripción corta</t>
+          <t>Detalle (texto largo)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Detalle (texto largo)</t>
+          <t>Talla</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Talla</t>
+          <t>Material</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
           <t>Colores (por nombre, separados por coma)</t>
         </is>
       </c>
-      <c r="K1" s="29" t="inlineStr">
+      <c r="J1" s="29" t="inlineStr">
         <is>
           <t>Nuevo (sí / no)</t>
         </is>
@@ -701,35 +696,30 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>boina.jpg, boina-2.jpg, boina-3.jpg</t>
+          <t>Boina tejida con lazo, suave y abrigadora.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Boina tejida con lazo, suave y abrigadora.</t>
+          <t>Boina tejida de punto suave que abriga sin apretar. El lazo va cosido a mano para que no se suelte. Ideal para fotos, paseos y ocasiones especiales.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Boina tejida de punto suave que abriga sin apretar. El lazo va cosido a mano para que no se suelte. Ideal para fotos, paseos y ocasiones especiales.</t>
+          <t>Talla única · 0 a 12 meses</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Talla única · 0 a 12 meses</t>
+          <t>Tejido acrílico suave</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Tejido acrílico suave</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
           <t>blanco, rojo, rosa, negro, beige, lila</t>
         </is>
       </c>
-      <c r="K2" s="30" t="inlineStr">
+      <c r="J2" s="30" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -752,31 +742,26 @@
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>pantys.jpg, pantys-2.jpg</t>
+          <t>Pantys de algodón con diseño de pandita.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Pantys de algodón con diseño de pandita.</t>
+          <t>Pantys de algodón con diseño de pandita en las rodillas. Tela elástica que no aprieta la barriguita.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Pantys de algodón con diseño de pandita en las rodillas. Tela elástica que no aprieta la barriguita.</t>
+          <t>Tallas 0 a 24 meses</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Tallas 0 a 24 meses</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
           <t>Algodón con elastano</t>
         </is>
       </c>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="30" t="inlineStr">
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="30" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -801,31 +786,26 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>lentes.jpg</t>
+          <t>Lentes con orejitas de gatito y protección UV.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Lentes con orejitas de gatito y protección UV.</t>
+          <t>Lentes de sol con orejitas de gatito y protección UV400. Montura flexible y resistente.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Lentes de sol con orejitas de gatito y protección UV400. Montura flexible y resistente.</t>
+          <t>Para niñas de 1 a 5 años</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Para niñas de 1 a 5 años</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
           <t>Marco flexible · UV400</t>
         </is>
       </c>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="30" t="inlineStr">
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="30" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
@@ -841,8 +821,7 @@
       <c r="G5" s="3" t="n"/>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="30" t="n"/>
+      <c r="J5" s="30" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n"/>
@@ -854,8 +833,7 @@
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="30" t="n"/>
+      <c r="J6" s="30" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n"/>
@@ -867,8 +845,7 @@
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="30" t="n"/>
+      <c r="J7" s="30" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
@@ -880,8 +857,7 @@
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="30" t="n"/>
+      <c r="J8" s="30" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n"/>
@@ -893,8 +869,7 @@
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="30" t="n"/>
+      <c r="J9" s="30" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
@@ -906,8 +881,7 @@
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="30" t="n"/>
+      <c r="J10" s="30" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>
@@ -919,8 +893,7 @@
       <c r="G11" s="3" t="n"/>
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="30" t="n"/>
+      <c r="J11" s="30" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
@@ -932,8 +905,7 @@
       <c r="G12" s="3" t="n"/>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="30" t="n"/>
+      <c r="J12" s="30" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -945,8 +917,7 @@
       <c r="G13" s="3" t="n"/>
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="30" t="n"/>
+      <c r="J13" s="30" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -958,8 +929,7 @@
       <c r="G14" s="3" t="n"/>
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="30" t="n"/>
+      <c r="J14" s="30" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
@@ -971,8 +941,7 @@
       <c r="G15" s="3" t="n"/>
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="3" t="n"/>
-      <c r="J15" s="3" t="n"/>
-      <c r="K15" s="30" t="n"/>
+      <c r="J15" s="30" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
@@ -984,8 +953,7 @@
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="3" t="n"/>
-      <c r="J16" s="3" t="n"/>
-      <c r="K16" s="30" t="n"/>
+      <c r="J16" s="30" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
@@ -997,8 +965,7 @@
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="3" t="n"/>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="30" t="n"/>
+      <c r="J17" s="30" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
@@ -1010,8 +977,7 @@
       <c r="G18" s="3" t="n"/>
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="3" t="n"/>
-      <c r="J18" s="3" t="n"/>
-      <c r="K18" s="30" t="n"/>
+      <c r="J18" s="30" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
@@ -1023,8 +989,7 @@
       <c r="G19" s="3" t="n"/>
       <c r="H19" s="3" t="n"/>
       <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="30" t="n"/>
+      <c r="J19" s="30" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
@@ -1036,8 +1001,7 @@
       <c r="G20" s="3" t="n"/>
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n"/>
-      <c r="J20" s="3" t="n"/>
-      <c r="K20" s="30" t="n"/>
+      <c r="J20" s="30" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
@@ -1049,8 +1013,7 @@
       <c r="G21" s="3" t="n"/>
       <c r="H21" s="3" t="n"/>
       <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="30" t="n"/>
+      <c r="J21" s="30" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
@@ -1062,8 +1025,7 @@
       <c r="G22" s="3" t="n"/>
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="30" t="n"/>
+      <c r="J22" s="30" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
@@ -1075,8 +1037,7 @@
       <c r="G23" s="3" t="n"/>
       <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="30" t="n"/>
+      <c r="J23" s="30" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
@@ -1088,8 +1049,7 @@
       <c r="G24" s="3" t="n"/>
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="30" t="n"/>
+      <c r="J24" s="30" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
@@ -1101,8 +1061,7 @@
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>
-      <c r="J25" s="3" t="n"/>
-      <c r="K25" s="30" t="n"/>
+      <c r="J25" s="30" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
@@ -1114,8 +1073,7 @@
       <c r="G26" s="3" t="n"/>
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
-      <c r="J26" s="3" t="n"/>
-      <c r="K26" s="30" t="n"/>
+      <c r="J26" s="30" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
@@ -1127,8 +1085,7 @@
       <c r="G27" s="3" t="n"/>
       <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="n"/>
-      <c r="J27" s="3" t="n"/>
-      <c r="K27" s="30" t="n"/>
+      <c r="J27" s="30" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
@@ -1140,8 +1097,7 @@
       <c r="G28" s="3" t="n"/>
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n"/>
-      <c r="J28" s="3" t="n"/>
-      <c r="K28" s="30" t="n"/>
+      <c r="J28" s="30" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
@@ -1153,8 +1109,7 @@
       <c r="G29" s="3" t="n"/>
       <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="n"/>
-      <c r="J29" s="3" t="n"/>
-      <c r="K29" s="30" t="n"/>
+      <c r="J29" s="30" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
@@ -1166,8 +1121,7 @@
       <c r="G30" s="3" t="n"/>
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n"/>
-      <c r="J30" s="3" t="n"/>
-      <c r="K30" s="30" t="n"/>
+      <c r="J30" s="30" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
@@ -1179,8 +1133,7 @@
       <c r="G31" s="3" t="n"/>
       <c r="H31" s="3" t="n"/>
       <c r="I31" s="3" t="n"/>
-      <c r="J31" s="3" t="n"/>
-      <c r="K31" s="30" t="n"/>
+      <c r="J31" s="30" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n"/>
@@ -1192,8 +1145,7 @@
       <c r="G32" s="3" t="n"/>
       <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="n"/>
-      <c r="J32" s="3" t="n"/>
-      <c r="K32" s="30" t="n"/>
+      <c r="J32" s="30" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n"/>
@@ -1205,8 +1157,7 @@
       <c r="G33" s="3" t="n"/>
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="n"/>
-      <c r="J33" s="3" t="n"/>
-      <c r="K33" s="30" t="n"/>
+      <c r="J33" s="30" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n"/>
@@ -1218,8 +1169,7 @@
       <c r="G34" s="3" t="n"/>
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
-      <c r="J34" s="3" t="n"/>
-      <c r="K34" s="30" t="n"/>
+      <c r="J34" s="30" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>
@@ -1231,8 +1181,7 @@
       <c r="G35" s="3" t="n"/>
       <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="n"/>
-      <c r="J35" s="3" t="n"/>
-      <c r="K35" s="30" t="n"/>
+      <c r="J35" s="30" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
@@ -1244,8 +1193,7 @@
       <c r="G36" s="3" t="n"/>
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
-      <c r="J36" s="3" t="n"/>
-      <c r="K36" s="30" t="n"/>
+      <c r="J36" s="30" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
@@ -1257,8 +1205,7 @@
       <c r="G37" s="3" t="n"/>
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="n"/>
-      <c r="J37" s="3" t="n"/>
-      <c r="K37" s="30" t="n"/>
+      <c r="J37" s="30" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
@@ -1270,8 +1217,7 @@
       <c r="G38" s="3" t="n"/>
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n"/>
-      <c r="J38" s="3" t="n"/>
-      <c r="K38" s="30" t="n"/>
+      <c r="J38" s="30" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
@@ -1283,8 +1229,7 @@
       <c r="G39" s="3" t="n"/>
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="n"/>
-      <c r="J39" s="3" t="n"/>
-      <c r="K39" s="30" t="n"/>
+      <c r="J39" s="30" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
@@ -1296,8 +1241,7 @@
       <c r="G40" s="3" t="n"/>
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n"/>
-      <c r="J40" s="3" t="n"/>
-      <c r="K40" s="30" t="n"/>
+      <c r="J40" s="30" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
@@ -1309,8 +1253,7 @@
       <c r="G41" s="3" t="n"/>
       <c r="H41" s="3" t="n"/>
       <c r="I41" s="3" t="n"/>
-      <c r="J41" s="3" t="n"/>
-      <c r="K41" s="30" t="n"/>
+      <c r="J41" s="30" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
@@ -1322,8 +1265,7 @@
       <c r="G42" s="3" t="n"/>
       <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="n"/>
-      <c r="J42" s="3" t="n"/>
-      <c r="K42" s="30" t="n"/>
+      <c r="J42" s="30" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
@@ -1335,8 +1277,7 @@
       <c r="G43" s="3" t="n"/>
       <c r="H43" s="3" t="n"/>
       <c r="I43" s="3" t="n"/>
-      <c r="J43" s="3" t="n"/>
-      <c r="K43" s="30" t="n"/>
+      <c r="J43" s="30" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
@@ -1348,8 +1289,7 @@
       <c r="G44" s="3" t="n"/>
       <c r="H44" s="3" t="n"/>
       <c r="I44" s="3" t="n"/>
-      <c r="J44" s="3" t="n"/>
-      <c r="K44" s="30" t="n"/>
+      <c r="J44" s="30" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
@@ -1361,8 +1301,7 @@
       <c r="G45" s="3" t="n"/>
       <c r="H45" s="3" t="n"/>
       <c r="I45" s="3" t="n"/>
-      <c r="J45" s="3" t="n"/>
-      <c r="K45" s="30" t="n"/>
+      <c r="J45" s="30" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
@@ -1374,8 +1313,7 @@
       <c r="G46" s="3" t="n"/>
       <c r="H46" s="3" t="n"/>
       <c r="I46" s="3" t="n"/>
-      <c r="J46" s="3" t="n"/>
-      <c r="K46" s="30" t="n"/>
+      <c r="J46" s="30" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
@@ -1387,8 +1325,7 @@
       <c r="G47" s="3" t="n"/>
       <c r="H47" s="3" t="n"/>
       <c r="I47" s="3" t="n"/>
-      <c r="J47" s="3" t="n"/>
-      <c r="K47" s="30" t="n"/>
+      <c r="J47" s="30" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -1400,8 +1337,7 @@
       <c r="G48" s="3" t="n"/>
       <c r="H48" s="3" t="n"/>
       <c r="I48" s="3" t="n"/>
-      <c r="J48" s="3" t="n"/>
-      <c r="K48" s="30" t="n"/>
+      <c r="J48" s="30" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
@@ -1413,8 +1349,7 @@
       <c r="G49" s="3" t="n"/>
       <c r="H49" s="3" t="n"/>
       <c r="I49" s="3" t="n"/>
-      <c r="J49" s="3" t="n"/>
-      <c r="K49" s="30" t="n"/>
+      <c r="J49" s="30" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
@@ -1426,8 +1361,7 @@
       <c r="G50" s="3" t="n"/>
       <c r="H50" s="3" t="n"/>
       <c r="I50" s="3" t="n"/>
-      <c r="J50" s="3" t="n"/>
-      <c r="K50" s="30" t="n"/>
+      <c r="J50" s="30" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
@@ -1439,8 +1373,7 @@
       <c r="G51" s="3" t="n"/>
       <c r="H51" s="3" t="n"/>
       <c r="I51" s="3" t="n"/>
-      <c r="J51" s="3" t="n"/>
-      <c r="K51" s="30" t="n"/>
+      <c r="J51" s="30" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
@@ -1452,8 +1385,7 @@
       <c r="G52" s="3" t="n"/>
       <c r="H52" s="3" t="n"/>
       <c r="I52" s="3" t="n"/>
-      <c r="J52" s="3" t="n"/>
-      <c r="K52" s="30" t="n"/>
+      <c r="J52" s="30" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n"/>
@@ -1465,8 +1397,7 @@
       <c r="G53" s="3" t="n"/>
       <c r="H53" s="3" t="n"/>
       <c r="I53" s="3" t="n"/>
-      <c r="J53" s="3" t="n"/>
-      <c r="K53" s="30" t="n"/>
+      <c r="J53" s="30" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
@@ -1478,8 +1409,7 @@
       <c r="G54" s="3" t="n"/>
       <c r="H54" s="3" t="n"/>
       <c r="I54" s="3" t="n"/>
-      <c r="J54" s="3" t="n"/>
-      <c r="K54" s="30" t="n"/>
+      <c r="J54" s="30" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
@@ -1491,8 +1421,7 @@
       <c r="G55" s="3" t="n"/>
       <c r="H55" s="3" t="n"/>
       <c r="I55" s="3" t="n"/>
-      <c r="J55" s="3" t="n"/>
-      <c r="K55" s="30" t="n"/>
+      <c r="J55" s="30" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
@@ -1504,8 +1433,7 @@
       <c r="G56" s="3" t="n"/>
       <c r="H56" s="3" t="n"/>
       <c r="I56" s="3" t="n"/>
-      <c r="J56" s="3" t="n"/>
-      <c r="K56" s="30" t="n"/>
+      <c r="J56" s="30" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
@@ -1517,8 +1445,7 @@
       <c r="G57" s="3" t="n"/>
       <c r="H57" s="3" t="n"/>
       <c r="I57" s="3" t="n"/>
-      <c r="J57" s="3" t="n"/>
-      <c r="K57" s="30" t="n"/>
+      <c r="J57" s="30" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
@@ -1530,8 +1457,7 @@
       <c r="G58" s="3" t="n"/>
       <c r="H58" s="3" t="n"/>
       <c r="I58" s="3" t="n"/>
-      <c r="J58" s="3" t="n"/>
-      <c r="K58" s="30" t="n"/>
+      <c r="J58" s="30" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
@@ -1543,8 +1469,7 @@
       <c r="G59" s="3" t="n"/>
       <c r="H59" s="3" t="n"/>
       <c r="I59" s="3" t="n"/>
-      <c r="J59" s="3" t="n"/>
-      <c r="K59" s="30" t="n"/>
+      <c r="J59" s="30" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
@@ -1556,8 +1481,7 @@
       <c r="G60" s="3" t="n"/>
       <c r="H60" s="3" t="n"/>
       <c r="I60" s="3" t="n"/>
-      <c r="J60" s="3" t="n"/>
-      <c r="K60" s="30" t="n"/>
+      <c r="J60" s="30" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
@@ -1569,8 +1493,7 @@
       <c r="G61" s="3" t="n"/>
       <c r="H61" s="3" t="n"/>
       <c r="I61" s="3" t="n"/>
-      <c r="J61" s="3" t="n"/>
-      <c r="K61" s="30" t="n"/>
+      <c r="J61" s="30" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
@@ -1582,8 +1505,7 @@
       <c r="G62" s="3" t="n"/>
       <c r="H62" s="3" t="n"/>
       <c r="I62" s="3" t="n"/>
-      <c r="J62" s="3" t="n"/>
-      <c r="K62" s="30" t="n"/>
+      <c r="J62" s="30" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>
@@ -1595,8 +1517,7 @@
       <c r="G63" s="3" t="n"/>
       <c r="H63" s="3" t="n"/>
       <c r="I63" s="3" t="n"/>
-      <c r="J63" s="3" t="n"/>
-      <c r="K63" s="30" t="n"/>
+      <c r="J63" s="30" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>
@@ -1608,8 +1529,7 @@
       <c r="G64" s="3" t="n"/>
       <c r="H64" s="3" t="n"/>
       <c r="I64" s="3" t="n"/>
-      <c r="J64" s="3" t="n"/>
-      <c r="K64" s="30" t="n"/>
+      <c r="J64" s="30" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
@@ -1621,8 +1541,7 @@
       <c r="G65" s="3" t="n"/>
       <c r="H65" s="3" t="n"/>
       <c r="I65" s="3" t="n"/>
-      <c r="J65" s="3" t="n"/>
-      <c r="K65" s="30" t="n"/>
+      <c r="J65" s="30" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
@@ -1634,8 +1553,7 @@
       <c r="G66" s="3" t="n"/>
       <c r="H66" s="3" t="n"/>
       <c r="I66" s="3" t="n"/>
-      <c r="J66" s="3" t="n"/>
-      <c r="K66" s="30" t="n"/>
+      <c r="J66" s="30" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
@@ -1647,8 +1565,7 @@
       <c r="G67" s="3" t="n"/>
       <c r="H67" s="3" t="n"/>
       <c r="I67" s="3" t="n"/>
-      <c r="J67" s="3" t="n"/>
-      <c r="K67" s="30" t="n"/>
+      <c r="J67" s="30" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n"/>
@@ -1660,8 +1577,7 @@
       <c r="G68" s="3" t="n"/>
       <c r="H68" s="3" t="n"/>
       <c r="I68" s="3" t="n"/>
-      <c r="J68" s="3" t="n"/>
-      <c r="K68" s="30" t="n"/>
+      <c r="J68" s="30" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
@@ -1673,8 +1589,7 @@
       <c r="G69" s="3" t="n"/>
       <c r="H69" s="3" t="n"/>
       <c r="I69" s="3" t="n"/>
-      <c r="J69" s="3" t="n"/>
-      <c r="K69" s="30" t="n"/>
+      <c r="J69" s="30" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
@@ -1686,8 +1601,7 @@
       <c r="G70" s="3" t="n"/>
       <c r="H70" s="3" t="n"/>
       <c r="I70" s="3" t="n"/>
-      <c r="J70" s="3" t="n"/>
-      <c r="K70" s="30" t="n"/>
+      <c r="J70" s="30" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
@@ -1699,8 +1613,7 @@
       <c r="G71" s="3" t="n"/>
       <c r="H71" s="3" t="n"/>
       <c r="I71" s="3" t="n"/>
-      <c r="J71" s="3" t="n"/>
-      <c r="K71" s="30" t="n"/>
+      <c r="J71" s="30" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
@@ -1712,8 +1625,7 @@
       <c r="G72" s="3" t="n"/>
       <c r="H72" s="3" t="n"/>
       <c r="I72" s="3" t="n"/>
-      <c r="J72" s="3" t="n"/>
-      <c r="K72" s="30" t="n"/>
+      <c r="J72" s="30" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
@@ -1725,8 +1637,7 @@
       <c r="G73" s="3" t="n"/>
       <c r="H73" s="3" t="n"/>
       <c r="I73" s="3" t="n"/>
-      <c r="J73" s="3" t="n"/>
-      <c r="K73" s="30" t="n"/>
+      <c r="J73" s="30" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
@@ -1738,8 +1649,7 @@
       <c r="G74" s="3" t="n"/>
       <c r="H74" s="3" t="n"/>
       <c r="I74" s="3" t="n"/>
-      <c r="J74" s="3" t="n"/>
-      <c r="K74" s="30" t="n"/>
+      <c r="J74" s="30" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
@@ -1751,8 +1661,7 @@
       <c r="G75" s="3" t="n"/>
       <c r="H75" s="3" t="n"/>
       <c r="I75" s="3" t="n"/>
-      <c r="J75" s="3" t="n"/>
-      <c r="K75" s="30" t="n"/>
+      <c r="J75" s="30" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n"/>
@@ -1764,8 +1673,7 @@
       <c r="G76" s="3" t="n"/>
       <c r="H76" s="3" t="n"/>
       <c r="I76" s="3" t="n"/>
-      <c r="J76" s="3" t="n"/>
-      <c r="K76" s="30" t="n"/>
+      <c r="J76" s="30" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
@@ -1777,8 +1685,7 @@
       <c r="G77" s="3" t="n"/>
       <c r="H77" s="3" t="n"/>
       <c r="I77" s="3" t="n"/>
-      <c r="J77" s="3" t="n"/>
-      <c r="K77" s="30" t="n"/>
+      <c r="J77" s="30" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
@@ -1790,8 +1697,7 @@
       <c r="G78" s="3" t="n"/>
       <c r="H78" s="3" t="n"/>
       <c r="I78" s="3" t="n"/>
-      <c r="J78" s="3" t="n"/>
-      <c r="K78" s="30" t="n"/>
+      <c r="J78" s="30" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
@@ -1803,8 +1709,7 @@
       <c r="G79" s="3" t="n"/>
       <c r="H79" s="3" t="n"/>
       <c r="I79" s="3" t="n"/>
-      <c r="J79" s="3" t="n"/>
-      <c r="K79" s="30" t="n"/>
+      <c r="J79" s="30" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
@@ -1816,8 +1721,7 @@
       <c r="G80" s="3" t="n"/>
       <c r="H80" s="3" t="n"/>
       <c r="I80" s="3" t="n"/>
-      <c r="J80" s="3" t="n"/>
-      <c r="K80" s="30" t="n"/>
+      <c r="J80" s="30" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
@@ -1829,8 +1733,7 @@
       <c r="G81" s="3" t="n"/>
       <c r="H81" s="3" t="n"/>
       <c r="I81" s="3" t="n"/>
-      <c r="J81" s="3" t="n"/>
-      <c r="K81" s="30" t="n"/>
+      <c r="J81" s="30" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
@@ -1842,8 +1745,7 @@
       <c r="G82" s="3" t="n"/>
       <c r="H82" s="3" t="n"/>
       <c r="I82" s="3" t="n"/>
-      <c r="J82" s="3" t="n"/>
-      <c r="K82" s="30" t="n"/>
+      <c r="J82" s="30" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
@@ -1855,8 +1757,7 @@
       <c r="G83" s="3" t="n"/>
       <c r="H83" s="3" t="n"/>
       <c r="I83" s="3" t="n"/>
-      <c r="J83" s="3" t="n"/>
-      <c r="K83" s="30" t="n"/>
+      <c r="J83" s="30" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
@@ -1868,8 +1769,7 @@
       <c r="G84" s="3" t="n"/>
       <c r="H84" s="3" t="n"/>
       <c r="I84" s="3" t="n"/>
-      <c r="J84" s="3" t="n"/>
-      <c r="K84" s="30" t="n"/>
+      <c r="J84" s="30" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n"/>
@@ -1881,8 +1781,7 @@
       <c r="G85" s="3" t="n"/>
       <c r="H85" s="3" t="n"/>
       <c r="I85" s="3" t="n"/>
-      <c r="J85" s="3" t="n"/>
-      <c r="K85" s="30" t="n"/>
+      <c r="J85" s="30" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n"/>
@@ -1894,8 +1793,7 @@
       <c r="G86" s="3" t="n"/>
       <c r="H86" s="3" t="n"/>
       <c r="I86" s="3" t="n"/>
-      <c r="J86" s="3" t="n"/>
-      <c r="K86" s="30" t="n"/>
+      <c r="J86" s="30" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n"/>
@@ -1907,8 +1805,7 @@
       <c r="G87" s="3" t="n"/>
       <c r="H87" s="3" t="n"/>
       <c r="I87" s="3" t="n"/>
-      <c r="J87" s="3" t="n"/>
-      <c r="K87" s="30" t="n"/>
+      <c r="J87" s="30" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
@@ -1920,8 +1817,7 @@
       <c r="G88" s="3" t="n"/>
       <c r="H88" s="3" t="n"/>
       <c r="I88" s="3" t="n"/>
-      <c r="J88" s="3" t="n"/>
-      <c r="K88" s="30" t="n"/>
+      <c r="J88" s="30" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n"/>
@@ -1933,8 +1829,7 @@
       <c r="G89" s="3" t="n"/>
       <c r="H89" s="3" t="n"/>
       <c r="I89" s="3" t="n"/>
-      <c r="J89" s="3" t="n"/>
-      <c r="K89" s="30" t="n"/>
+      <c r="J89" s="30" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n"/>
@@ -1946,8 +1841,7 @@
       <c r="G90" s="3" t="n"/>
       <c r="H90" s="3" t="n"/>
       <c r="I90" s="3" t="n"/>
-      <c r="J90" s="3" t="n"/>
-      <c r="K90" s="30" t="n"/>
+      <c r="J90" s="30" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n"/>
@@ -1959,8 +1853,7 @@
       <c r="G91" s="3" t="n"/>
       <c r="H91" s="3" t="n"/>
       <c r="I91" s="3" t="n"/>
-      <c r="J91" s="3" t="n"/>
-      <c r="K91" s="30" t="n"/>
+      <c r="J91" s="30" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n"/>
@@ -1972,8 +1865,7 @@
       <c r="G92" s="3" t="n"/>
       <c r="H92" s="3" t="n"/>
       <c r="I92" s="3" t="n"/>
-      <c r="J92" s="3" t="n"/>
-      <c r="K92" s="30" t="n"/>
+      <c r="J92" s="30" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n"/>
@@ -1985,8 +1877,7 @@
       <c r="G93" s="3" t="n"/>
       <c r="H93" s="3" t="n"/>
       <c r="I93" s="3" t="n"/>
-      <c r="J93" s="3" t="n"/>
-      <c r="K93" s="30" t="n"/>
+      <c r="J93" s="30" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n"/>
@@ -1998,8 +1889,7 @@
       <c r="G94" s="3" t="n"/>
       <c r="H94" s="3" t="n"/>
       <c r="I94" s="3" t="n"/>
-      <c r="J94" s="3" t="n"/>
-      <c r="K94" s="30" t="n"/>
+      <c r="J94" s="30" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n"/>
@@ -2011,8 +1901,7 @@
       <c r="G95" s="3" t="n"/>
       <c r="H95" s="3" t="n"/>
       <c r="I95" s="3" t="n"/>
-      <c r="J95" s="3" t="n"/>
-      <c r="K95" s="30" t="n"/>
+      <c r="J95" s="30" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n"/>
@@ -2024,8 +1913,7 @@
       <c r="G96" s="3" t="n"/>
       <c r="H96" s="3" t="n"/>
       <c r="I96" s="3" t="n"/>
-      <c r="J96" s="3" t="n"/>
-      <c r="K96" s="30" t="n"/>
+      <c r="J96" s="30" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n"/>
@@ -2037,8 +1925,7 @@
       <c r="G97" s="3" t="n"/>
       <c r="H97" s="3" t="n"/>
       <c r="I97" s="3" t="n"/>
-      <c r="J97" s="3" t="n"/>
-      <c r="K97" s="30" t="n"/>
+      <c r="J97" s="30" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n"/>
@@ -2050,8 +1937,7 @@
       <c r="G98" s="3" t="n"/>
       <c r="H98" s="3" t="n"/>
       <c r="I98" s="3" t="n"/>
-      <c r="J98" s="3" t="n"/>
-      <c r="K98" s="30" t="n"/>
+      <c r="J98" s="30" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n"/>
@@ -2063,8 +1949,7 @@
       <c r="G99" s="3" t="n"/>
       <c r="H99" s="3" t="n"/>
       <c r="I99" s="3" t="n"/>
-      <c r="J99" s="3" t="n"/>
-      <c r="K99" s="30" t="n"/>
+      <c r="J99" s="30" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n"/>
@@ -2076,8 +1961,7 @@
       <c r="G100" s="3" t="n"/>
       <c r="H100" s="3" t="n"/>
       <c r="I100" s="3" t="n"/>
-      <c r="J100" s="3" t="n"/>
-      <c r="K100" s="30" t="n"/>
+      <c r="J100" s="30" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n"/>
@@ -2089,8 +1973,7 @@
       <c r="G101" s="3" t="n"/>
       <c r="H101" s="3" t="n"/>
       <c r="I101" s="3" t="n"/>
-      <c r="J101" s="3" t="n"/>
-      <c r="K101" s="30" t="n"/>
+      <c r="J101" s="30" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n"/>
@@ -2102,8 +1985,7 @@
       <c r="G102" s="3" t="n"/>
       <c r="H102" s="3" t="n"/>
       <c r="I102" s="3" t="n"/>
-      <c r="J102" s="3" t="n"/>
-      <c r="K102" s="30" t="n"/>
+      <c r="J102" s="30" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n"/>
@@ -2115,8 +1997,7 @@
       <c r="G103" s="3" t="n"/>
       <c r="H103" s="3" t="n"/>
       <c r="I103" s="3" t="n"/>
-      <c r="J103" s="3" t="n"/>
-      <c r="K103" s="30" t="n"/>
+      <c r="J103" s="30" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n"/>
@@ -2128,8 +2009,7 @@
       <c r="G104" s="3" t="n"/>
       <c r="H104" s="3" t="n"/>
       <c r="I104" s="3" t="n"/>
-      <c r="J104" s="3" t="n"/>
-      <c r="K104" s="30" t="n"/>
+      <c r="J104" s="30" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n"/>
@@ -2141,8 +2021,7 @@
       <c r="G105" s="3" t="n"/>
       <c r="H105" s="3" t="n"/>
       <c r="I105" s="3" t="n"/>
-      <c r="J105" s="3" t="n"/>
-      <c r="K105" s="30" t="n"/>
+      <c r="J105" s="30" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n"/>
@@ -2154,8 +2033,7 @@
       <c r="G106" s="3" t="n"/>
       <c r="H106" s="3" t="n"/>
       <c r="I106" s="3" t="n"/>
-      <c r="J106" s="3" t="n"/>
-      <c r="K106" s="30" t="n"/>
+      <c r="J106" s="30" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n"/>
@@ -2167,8 +2045,7 @@
       <c r="G107" s="3" t="n"/>
       <c r="H107" s="3" t="n"/>
       <c r="I107" s="3" t="n"/>
-      <c r="J107" s="3" t="n"/>
-      <c r="K107" s="30" t="n"/>
+      <c r="J107" s="30" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n"/>
@@ -2180,8 +2057,7 @@
       <c r="G108" s="3" t="n"/>
       <c r="H108" s="3" t="n"/>
       <c r="I108" s="3" t="n"/>
-      <c r="J108" s="3" t="n"/>
-      <c r="K108" s="30" t="n"/>
+      <c r="J108" s="30" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n"/>
@@ -2193,8 +2069,7 @@
       <c r="G109" s="3" t="n"/>
       <c r="H109" s="3" t="n"/>
       <c r="I109" s="3" t="n"/>
-      <c r="J109" s="3" t="n"/>
-      <c r="K109" s="30" t="n"/>
+      <c r="J109" s="30" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n"/>
@@ -2206,8 +2081,7 @@
       <c r="G110" s="3" t="n"/>
       <c r="H110" s="3" t="n"/>
       <c r="I110" s="3" t="n"/>
-      <c r="J110" s="3" t="n"/>
-      <c r="K110" s="30" t="n"/>
+      <c r="J110" s="30" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n"/>
@@ -2219,8 +2093,7 @@
       <c r="G111" s="3" t="n"/>
       <c r="H111" s="3" t="n"/>
       <c r="I111" s="3" t="n"/>
-      <c r="J111" s="3" t="n"/>
-      <c r="K111" s="30" t="n"/>
+      <c r="J111" s="30" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n"/>
@@ -2232,8 +2105,7 @@
       <c r="G112" s="3" t="n"/>
       <c r="H112" s="3" t="n"/>
       <c r="I112" s="3" t="n"/>
-      <c r="J112" s="3" t="n"/>
-      <c r="K112" s="30" t="n"/>
+      <c r="J112" s="30" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n"/>
@@ -2245,8 +2117,7 @@
       <c r="G113" s="3" t="n"/>
       <c r="H113" s="3" t="n"/>
       <c r="I113" s="3" t="n"/>
-      <c r="J113" s="3" t="n"/>
-      <c r="K113" s="30" t="n"/>
+      <c r="J113" s="30" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n"/>
@@ -2258,8 +2129,7 @@
       <c r="G114" s="3" t="n"/>
       <c r="H114" s="3" t="n"/>
       <c r="I114" s="3" t="n"/>
-      <c r="J114" s="3" t="n"/>
-      <c r="K114" s="30" t="n"/>
+      <c r="J114" s="30" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n"/>
@@ -2271,8 +2141,7 @@
       <c r="G115" s="3" t="n"/>
       <c r="H115" s="3" t="n"/>
       <c r="I115" s="3" t="n"/>
-      <c r="J115" s="3" t="n"/>
-      <c r="K115" s="30" t="n"/>
+      <c r="J115" s="30" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n"/>
@@ -2284,8 +2153,7 @@
       <c r="G116" s="3" t="n"/>
       <c r="H116" s="3" t="n"/>
       <c r="I116" s="3" t="n"/>
-      <c r="J116" s="3" t="n"/>
-      <c r="K116" s="30" t="n"/>
+      <c r="J116" s="30" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n"/>
@@ -2297,8 +2165,7 @@
       <c r="G117" s="3" t="n"/>
       <c r="H117" s="3" t="n"/>
       <c r="I117" s="3" t="n"/>
-      <c r="J117" s="3" t="n"/>
-      <c r="K117" s="30" t="n"/>
+      <c r="J117" s="30" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n"/>
@@ -2310,8 +2177,7 @@
       <c r="G118" s="3" t="n"/>
       <c r="H118" s="3" t="n"/>
       <c r="I118" s="3" t="n"/>
-      <c r="J118" s="3" t="n"/>
-      <c r="K118" s="30" t="n"/>
+      <c r="J118" s="30" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n"/>
@@ -2323,8 +2189,7 @@
       <c r="G119" s="3" t="n"/>
       <c r="H119" s="3" t="n"/>
       <c r="I119" s="3" t="n"/>
-      <c r="J119" s="3" t="n"/>
-      <c r="K119" s="30" t="n"/>
+      <c r="J119" s="30" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n"/>
@@ -2336,8 +2201,7 @@
       <c r="G120" s="3" t="n"/>
       <c r="H120" s="3" t="n"/>
       <c r="I120" s="3" t="n"/>
-      <c r="J120" s="3" t="n"/>
-      <c r="K120" s="30" t="n"/>
+      <c r="J120" s="30" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n"/>
@@ -2349,8 +2213,7 @@
       <c r="G121" s="3" t="n"/>
       <c r="H121" s="3" t="n"/>
       <c r="I121" s="3" t="n"/>
-      <c r="J121" s="3" t="n"/>
-      <c r="K121" s="30" t="n"/>
+      <c r="J121" s="30" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n"/>
@@ -2362,8 +2225,7 @@
       <c r="G122" s="3" t="n"/>
       <c r="H122" s="3" t="n"/>
       <c r="I122" s="3" t="n"/>
-      <c r="J122" s="3" t="n"/>
-      <c r="K122" s="30" t="n"/>
+      <c r="J122" s="30" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n"/>
@@ -2375,8 +2237,7 @@
       <c r="G123" s="3" t="n"/>
       <c r="H123" s="3" t="n"/>
       <c r="I123" s="3" t="n"/>
-      <c r="J123" s="3" t="n"/>
-      <c r="K123" s="30" t="n"/>
+      <c r="J123" s="30" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n"/>
@@ -2388,8 +2249,7 @@
       <c r="G124" s="3" t="n"/>
       <c r="H124" s="3" t="n"/>
       <c r="I124" s="3" t="n"/>
-      <c r="J124" s="3" t="n"/>
-      <c r="K124" s="30" t="n"/>
+      <c r="J124" s="30" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n"/>
@@ -2401,8 +2261,7 @@
       <c r="G125" s="3" t="n"/>
       <c r="H125" s="3" t="n"/>
       <c r="I125" s="3" t="n"/>
-      <c r="J125" s="3" t="n"/>
-      <c r="K125" s="30" t="n"/>
+      <c r="J125" s="30" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n"/>
@@ -2414,8 +2273,7 @@
       <c r="G126" s="3" t="n"/>
       <c r="H126" s="3" t="n"/>
       <c r="I126" s="3" t="n"/>
-      <c r="J126" s="3" t="n"/>
-      <c r="K126" s="30" t="n"/>
+      <c r="J126" s="30" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n"/>
@@ -2427,8 +2285,7 @@
       <c r="G127" s="3" t="n"/>
       <c r="H127" s="3" t="n"/>
       <c r="I127" s="3" t="n"/>
-      <c r="J127" s="3" t="n"/>
-      <c r="K127" s="30" t="n"/>
+      <c r="J127" s="30" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n"/>
@@ -2440,8 +2297,7 @@
       <c r="G128" s="3" t="n"/>
       <c r="H128" s="3" t="n"/>
       <c r="I128" s="3" t="n"/>
-      <c r="J128" s="3" t="n"/>
-      <c r="K128" s="30" t="n"/>
+      <c r="J128" s="30" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n"/>
@@ -2453,8 +2309,7 @@
       <c r="G129" s="3" t="n"/>
       <c r="H129" s="3" t="n"/>
       <c r="I129" s="3" t="n"/>
-      <c r="J129" s="3" t="n"/>
-      <c r="K129" s="30" t="n"/>
+      <c r="J129" s="30" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n"/>
@@ -2466,8 +2321,7 @@
       <c r="G130" s="3" t="n"/>
       <c r="H130" s="3" t="n"/>
       <c r="I130" s="3" t="n"/>
-      <c r="J130" s="3" t="n"/>
-      <c r="K130" s="30" t="n"/>
+      <c r="J130" s="30" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n"/>
@@ -2479,8 +2333,7 @@
       <c r="G131" s="3" t="n"/>
       <c r="H131" s="3" t="n"/>
       <c r="I131" s="3" t="n"/>
-      <c r="J131" s="3" t="n"/>
-      <c r="K131" s="30" t="n"/>
+      <c r="J131" s="30" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n"/>
@@ -2492,8 +2345,7 @@
       <c r="G132" s="3" t="n"/>
       <c r="H132" s="3" t="n"/>
       <c r="I132" s="3" t="n"/>
-      <c r="J132" s="3" t="n"/>
-      <c r="K132" s="30" t="n"/>
+      <c r="J132" s="30" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n"/>
@@ -2505,8 +2357,7 @@
       <c r="G133" s="3" t="n"/>
       <c r="H133" s="3" t="n"/>
       <c r="I133" s="3" t="n"/>
-      <c r="J133" s="3" t="n"/>
-      <c r="K133" s="30" t="n"/>
+      <c r="J133" s="30" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n"/>
@@ -2518,8 +2369,7 @@
       <c r="G134" s="3" t="n"/>
       <c r="H134" s="3" t="n"/>
       <c r="I134" s="3" t="n"/>
-      <c r="J134" s="3" t="n"/>
-      <c r="K134" s="30" t="n"/>
+      <c r="J134" s="30" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n"/>
@@ -2531,8 +2381,7 @@
       <c r="G135" s="3" t="n"/>
       <c r="H135" s="3" t="n"/>
       <c r="I135" s="3" t="n"/>
-      <c r="J135" s="3" t="n"/>
-      <c r="K135" s="30" t="n"/>
+      <c r="J135" s="30" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n"/>
@@ -2544,8 +2393,7 @@
       <c r="G136" s="3" t="n"/>
       <c r="H136" s="3" t="n"/>
       <c r="I136" s="3" t="n"/>
-      <c r="J136" s="3" t="n"/>
-      <c r="K136" s="30" t="n"/>
+      <c r="J136" s="30" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n"/>
@@ -2557,8 +2405,7 @@
       <c r="G137" s="3" t="n"/>
       <c r="H137" s="3" t="n"/>
       <c r="I137" s="3" t="n"/>
-      <c r="J137" s="3" t="n"/>
-      <c r="K137" s="30" t="n"/>
+      <c r="J137" s="30" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n"/>
@@ -2570,8 +2417,7 @@
       <c r="G138" s="3" t="n"/>
       <c r="H138" s="3" t="n"/>
       <c r="I138" s="3" t="n"/>
-      <c r="J138" s="3" t="n"/>
-      <c r="K138" s="30" t="n"/>
+      <c r="J138" s="30" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n"/>
@@ -2583,8 +2429,7 @@
       <c r="G139" s="3" t="n"/>
       <c r="H139" s="3" t="n"/>
       <c r="I139" s="3" t="n"/>
-      <c r="J139" s="3" t="n"/>
-      <c r="K139" s="30" t="n"/>
+      <c r="J139" s="30" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n"/>
@@ -2596,8 +2441,7 @@
       <c r="G140" s="3" t="n"/>
       <c r="H140" s="3" t="n"/>
       <c r="I140" s="3" t="n"/>
-      <c r="J140" s="3" t="n"/>
-      <c r="K140" s="30" t="n"/>
+      <c r="J140" s="30" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n"/>
@@ -2609,8 +2453,7 @@
       <c r="G141" s="3" t="n"/>
       <c r="H141" s="3" t="n"/>
       <c r="I141" s="3" t="n"/>
-      <c r="J141" s="3" t="n"/>
-      <c r="K141" s="30" t="n"/>
+      <c r="J141" s="30" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n"/>
@@ -2622,8 +2465,7 @@
       <c r="G142" s="3" t="n"/>
       <c r="H142" s="3" t="n"/>
       <c r="I142" s="3" t="n"/>
-      <c r="J142" s="3" t="n"/>
-      <c r="K142" s="30" t="n"/>
+      <c r="J142" s="30" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n"/>
@@ -2635,8 +2477,7 @@
       <c r="G143" s="3" t="n"/>
       <c r="H143" s="3" t="n"/>
       <c r="I143" s="3" t="n"/>
-      <c r="J143" s="3" t="n"/>
-      <c r="K143" s="30" t="n"/>
+      <c r="J143" s="30" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n"/>
@@ -2648,8 +2489,7 @@
       <c r="G144" s="3" t="n"/>
       <c r="H144" s="3" t="n"/>
       <c r="I144" s="3" t="n"/>
-      <c r="J144" s="3" t="n"/>
-      <c r="K144" s="30" t="n"/>
+      <c r="J144" s="30" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n"/>
@@ -2661,8 +2501,7 @@
       <c r="G145" s="3" t="n"/>
       <c r="H145" s="3" t="n"/>
       <c r="I145" s="3" t="n"/>
-      <c r="J145" s="3" t="n"/>
-      <c r="K145" s="30" t="n"/>
+      <c r="J145" s="30" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n"/>
@@ -2674,8 +2513,7 @@
       <c r="G146" s="3" t="n"/>
       <c r="H146" s="3" t="n"/>
       <c r="I146" s="3" t="n"/>
-      <c r="J146" s="3" t="n"/>
-      <c r="K146" s="30" t="n"/>
+      <c r="J146" s="30" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n"/>
@@ -2687,8 +2525,7 @@
       <c r="G147" s="3" t="n"/>
       <c r="H147" s="3" t="n"/>
       <c r="I147" s="3" t="n"/>
-      <c r="J147" s="3" t="n"/>
-      <c r="K147" s="30" t="n"/>
+      <c r="J147" s="30" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n"/>
@@ -2700,8 +2537,7 @@
       <c r="G148" s="3" t="n"/>
       <c r="H148" s="3" t="n"/>
       <c r="I148" s="3" t="n"/>
-      <c r="J148" s="3" t="n"/>
-      <c r="K148" s="30" t="n"/>
+      <c r="J148" s="30" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n"/>
@@ -2713,8 +2549,7 @@
       <c r="G149" s="3" t="n"/>
       <c r="H149" s="3" t="n"/>
       <c r="I149" s="3" t="n"/>
-      <c r="J149" s="3" t="n"/>
-      <c r="K149" s="30" t="n"/>
+      <c r="J149" s="30" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n"/>
@@ -2726,8 +2561,7 @@
       <c r="G150" s="3" t="n"/>
       <c r="H150" s="3" t="n"/>
       <c r="I150" s="3" t="n"/>
-      <c r="J150" s="3" t="n"/>
-      <c r="K150" s="30" t="n"/>
+      <c r="J150" s="30" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n"/>
@@ -2739,8 +2573,7 @@
       <c r="G151" s="3" t="n"/>
       <c r="H151" s="3" t="n"/>
       <c r="I151" s="3" t="n"/>
-      <c r="J151" s="3" t="n"/>
-      <c r="K151" s="30" t="n"/>
+      <c r="J151" s="30" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n"/>
@@ -2752,8 +2585,7 @@
       <c r="G152" s="3" t="n"/>
       <c r="H152" s="3" t="n"/>
       <c r="I152" s="3" t="n"/>
-      <c r="J152" s="3" t="n"/>
-      <c r="K152" s="30" t="n"/>
+      <c r="J152" s="30" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="n"/>
@@ -2765,8 +2597,7 @@
       <c r="G153" s="3" t="n"/>
       <c r="H153" s="3" t="n"/>
       <c r="I153" s="3" t="n"/>
-      <c r="J153" s="3" t="n"/>
-      <c r="K153" s="30" t="n"/>
+      <c r="J153" s="30" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n"/>
@@ -2778,8 +2609,7 @@
       <c r="G154" s="3" t="n"/>
       <c r="H154" s="3" t="n"/>
       <c r="I154" s="3" t="n"/>
-      <c r="J154" s="3" t="n"/>
-      <c r="K154" s="30" t="n"/>
+      <c r="J154" s="30" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n"/>
@@ -2791,8 +2621,7 @@
       <c r="G155" s="3" t="n"/>
       <c r="H155" s="3" t="n"/>
       <c r="I155" s="3" t="n"/>
-      <c r="J155" s="3" t="n"/>
-      <c r="K155" s="30" t="n"/>
+      <c r="J155" s="30" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n"/>
@@ -2804,8 +2633,7 @@
       <c r="G156" s="3" t="n"/>
       <c r="H156" s="3" t="n"/>
       <c r="I156" s="3" t="n"/>
-      <c r="J156" s="3" t="n"/>
-      <c r="K156" s="30" t="n"/>
+      <c r="J156" s="30" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n"/>
@@ -2817,8 +2645,7 @@
       <c r="G157" s="3" t="n"/>
       <c r="H157" s="3" t="n"/>
       <c r="I157" s="3" t="n"/>
-      <c r="J157" s="3" t="n"/>
-      <c r="K157" s="30" t="n"/>
+      <c r="J157" s="30" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n"/>
@@ -2830,8 +2657,7 @@
       <c r="G158" s="3" t="n"/>
       <c r="H158" s="3" t="n"/>
       <c r="I158" s="3" t="n"/>
-      <c r="J158" s="3" t="n"/>
-      <c r="K158" s="30" t="n"/>
+      <c r="J158" s="30" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n"/>
@@ -2843,8 +2669,7 @@
       <c r="G159" s="3" t="n"/>
       <c r="H159" s="3" t="n"/>
       <c r="I159" s="3" t="n"/>
-      <c r="J159" s="3" t="n"/>
-      <c r="K159" s="30" t="n"/>
+      <c r="J159" s="30" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n"/>
@@ -2856,8 +2681,7 @@
       <c r="G160" s="3" t="n"/>
       <c r="H160" s="3" t="n"/>
       <c r="I160" s="3" t="n"/>
-      <c r="J160" s="3" t="n"/>
-      <c r="K160" s="30" t="n"/>
+      <c r="J160" s="30" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="n"/>
@@ -2869,8 +2693,7 @@
       <c r="G161" s="3" t="n"/>
       <c r="H161" s="3" t="n"/>
       <c r="I161" s="3" t="n"/>
-      <c r="J161" s="3" t="n"/>
-      <c r="K161" s="30" t="n"/>
+      <c r="J161" s="30" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n"/>
@@ -2882,8 +2705,7 @@
       <c r="G162" s="3" t="n"/>
       <c r="H162" s="3" t="n"/>
       <c r="I162" s="3" t="n"/>
-      <c r="J162" s="3" t="n"/>
-      <c r="K162" s="30" t="n"/>
+      <c r="J162" s="30" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n"/>
@@ -2895,8 +2717,7 @@
       <c r="G163" s="3" t="n"/>
       <c r="H163" s="3" t="n"/>
       <c r="I163" s="3" t="n"/>
-      <c r="J163" s="3" t="n"/>
-      <c r="K163" s="30" t="n"/>
+      <c r="J163" s="30" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n"/>
@@ -2908,8 +2729,7 @@
       <c r="G164" s="3" t="n"/>
       <c r="H164" s="3" t="n"/>
       <c r="I164" s="3" t="n"/>
-      <c r="J164" s="3" t="n"/>
-      <c r="K164" s="30" t="n"/>
+      <c r="J164" s="30" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n"/>
@@ -2921,8 +2741,7 @@
       <c r="G165" s="3" t="n"/>
       <c r="H165" s="3" t="n"/>
       <c r="I165" s="3" t="n"/>
-      <c r="J165" s="3" t="n"/>
-      <c r="K165" s="30" t="n"/>
+      <c r="J165" s="30" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n"/>
@@ -2934,8 +2753,7 @@
       <c r="G166" s="3" t="n"/>
       <c r="H166" s="3" t="n"/>
       <c r="I166" s="3" t="n"/>
-      <c r="J166" s="3" t="n"/>
-      <c r="K166" s="30" t="n"/>
+      <c r="J166" s="30" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n"/>
@@ -2947,8 +2765,7 @@
       <c r="G167" s="3" t="n"/>
       <c r="H167" s="3" t="n"/>
       <c r="I167" s="3" t="n"/>
-      <c r="J167" s="3" t="n"/>
-      <c r="K167" s="30" t="n"/>
+      <c r="J167" s="30" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n"/>
@@ -2960,8 +2777,7 @@
       <c r="G168" s="3" t="n"/>
       <c r="H168" s="3" t="n"/>
       <c r="I168" s="3" t="n"/>
-      <c r="J168" s="3" t="n"/>
-      <c r="K168" s="30" t="n"/>
+      <c r="J168" s="30" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n"/>
@@ -2973,8 +2789,7 @@
       <c r="G169" s="3" t="n"/>
       <c r="H169" s="3" t="n"/>
       <c r="I169" s="3" t="n"/>
-      <c r="J169" s="3" t="n"/>
-      <c r="K169" s="30" t="n"/>
+      <c r="J169" s="30" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n"/>
@@ -2986,8 +2801,7 @@
       <c r="G170" s="3" t="n"/>
       <c r="H170" s="3" t="n"/>
       <c r="I170" s="3" t="n"/>
-      <c r="J170" s="3" t="n"/>
-      <c r="K170" s="30" t="n"/>
+      <c r="J170" s="30" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n"/>
@@ -2999,8 +2813,7 @@
       <c r="G171" s="3" t="n"/>
       <c r="H171" s="3" t="n"/>
       <c r="I171" s="3" t="n"/>
-      <c r="J171" s="3" t="n"/>
-      <c r="K171" s="30" t="n"/>
+      <c r="J171" s="30" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n"/>
@@ -3012,8 +2825,7 @@
       <c r="G172" s="3" t="n"/>
       <c r="H172" s="3" t="n"/>
       <c r="I172" s="3" t="n"/>
-      <c r="J172" s="3" t="n"/>
-      <c r="K172" s="30" t="n"/>
+      <c r="J172" s="30" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n"/>
@@ -3025,8 +2837,7 @@
       <c r="G173" s="3" t="n"/>
       <c r="H173" s="3" t="n"/>
       <c r="I173" s="3" t="n"/>
-      <c r="J173" s="3" t="n"/>
-      <c r="K173" s="30" t="n"/>
+      <c r="J173" s="30" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n"/>
@@ -3038,8 +2849,7 @@
       <c r="G174" s="3" t="n"/>
       <c r="H174" s="3" t="n"/>
       <c r="I174" s="3" t="n"/>
-      <c r="J174" s="3" t="n"/>
-      <c r="K174" s="30" t="n"/>
+      <c r="J174" s="30" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n"/>
@@ -3051,8 +2861,7 @@
       <c r="G175" s="3" t="n"/>
       <c r="H175" s="3" t="n"/>
       <c r="I175" s="3" t="n"/>
-      <c r="J175" s="3" t="n"/>
-      <c r="K175" s="30" t="n"/>
+      <c r="J175" s="30" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n"/>
@@ -3064,8 +2873,7 @@
       <c r="G176" s="3" t="n"/>
       <c r="H176" s="3" t="n"/>
       <c r="I176" s="3" t="n"/>
-      <c r="J176" s="3" t="n"/>
-      <c r="K176" s="30" t="n"/>
+      <c r="J176" s="30" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n"/>
@@ -3077,8 +2885,7 @@
       <c r="G177" s="3" t="n"/>
       <c r="H177" s="3" t="n"/>
       <c r="I177" s="3" t="n"/>
-      <c r="J177" s="3" t="n"/>
-      <c r="K177" s="30" t="n"/>
+      <c r="J177" s="30" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n"/>
@@ -3090,8 +2897,7 @@
       <c r="G178" s="3" t="n"/>
       <c r="H178" s="3" t="n"/>
       <c r="I178" s="3" t="n"/>
-      <c r="J178" s="3" t="n"/>
-      <c r="K178" s="30" t="n"/>
+      <c r="J178" s="30" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n"/>
@@ -3103,8 +2909,7 @@
       <c r="G179" s="3" t="n"/>
       <c r="H179" s="3" t="n"/>
       <c r="I179" s="3" t="n"/>
-      <c r="J179" s="3" t="n"/>
-      <c r="K179" s="30" t="n"/>
+      <c r="J179" s="30" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n"/>
@@ -3116,8 +2921,7 @@
       <c r="G180" s="3" t="n"/>
       <c r="H180" s="3" t="n"/>
       <c r="I180" s="3" t="n"/>
-      <c r="J180" s="3" t="n"/>
-      <c r="K180" s="30" t="n"/>
+      <c r="J180" s="30" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n"/>
@@ -3129,8 +2933,7 @@
       <c r="G181" s="3" t="n"/>
       <c r="H181" s="3" t="n"/>
       <c r="I181" s="3" t="n"/>
-      <c r="J181" s="3" t="n"/>
-      <c r="K181" s="30" t="n"/>
+      <c r="J181" s="30" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n"/>
@@ -3142,8 +2945,7 @@
       <c r="G182" s="3" t="n"/>
       <c r="H182" s="3" t="n"/>
       <c r="I182" s="3" t="n"/>
-      <c r="J182" s="3" t="n"/>
-      <c r="K182" s="30" t="n"/>
+      <c r="J182" s="30" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n"/>
@@ -3155,8 +2957,7 @@
       <c r="G183" s="3" t="n"/>
       <c r="H183" s="3" t="n"/>
       <c r="I183" s="3" t="n"/>
-      <c r="J183" s="3" t="n"/>
-      <c r="K183" s="30" t="n"/>
+      <c r="J183" s="30" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n"/>
@@ -3168,8 +2969,7 @@
       <c r="G184" s="3" t="n"/>
       <c r="H184" s="3" t="n"/>
       <c r="I184" s="3" t="n"/>
-      <c r="J184" s="3" t="n"/>
-      <c r="K184" s="30" t="n"/>
+      <c r="J184" s="30" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n"/>
@@ -3181,8 +2981,7 @@
       <c r="G185" s="3" t="n"/>
       <c r="H185" s="3" t="n"/>
       <c r="I185" s="3" t="n"/>
-      <c r="J185" s="3" t="n"/>
-      <c r="K185" s="30" t="n"/>
+      <c r="J185" s="30" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n"/>
@@ -3194,8 +2993,7 @@
       <c r="G186" s="3" t="n"/>
       <c r="H186" s="3" t="n"/>
       <c r="I186" s="3" t="n"/>
-      <c r="J186" s="3" t="n"/>
-      <c r="K186" s="30" t="n"/>
+      <c r="J186" s="30" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n"/>
@@ -3207,8 +3005,7 @@
       <c r="G187" s="3" t="n"/>
       <c r="H187" s="3" t="n"/>
       <c r="I187" s="3" t="n"/>
-      <c r="J187" s="3" t="n"/>
-      <c r="K187" s="30" t="n"/>
+      <c r="J187" s="30" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n"/>
@@ -3220,8 +3017,7 @@
       <c r="G188" s="3" t="n"/>
       <c r="H188" s="3" t="n"/>
       <c r="I188" s="3" t="n"/>
-      <c r="J188" s="3" t="n"/>
-      <c r="K188" s="30" t="n"/>
+      <c r="J188" s="30" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n"/>
@@ -3233,8 +3029,7 @@
       <c r="G189" s="3" t="n"/>
       <c r="H189" s="3" t="n"/>
       <c r="I189" s="3" t="n"/>
-      <c r="J189" s="3" t="n"/>
-      <c r="K189" s="30" t="n"/>
+      <c r="J189" s="30" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n"/>
@@ -3246,8 +3041,7 @@
       <c r="G190" s="3" t="n"/>
       <c r="H190" s="3" t="n"/>
       <c r="I190" s="3" t="n"/>
-      <c r="J190" s="3" t="n"/>
-      <c r="K190" s="30" t="n"/>
+      <c r="J190" s="30" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n"/>
@@ -3259,8 +3053,7 @@
       <c r="G191" s="3" t="n"/>
       <c r="H191" s="3" t="n"/>
       <c r="I191" s="3" t="n"/>
-      <c r="J191" s="3" t="n"/>
-      <c r="K191" s="30" t="n"/>
+      <c r="J191" s="30" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n"/>
@@ -3272,8 +3065,7 @@
       <c r="G192" s="3" t="n"/>
       <c r="H192" s="3" t="n"/>
       <c r="I192" s="3" t="n"/>
-      <c r="J192" s="3" t="n"/>
-      <c r="K192" s="30" t="n"/>
+      <c r="J192" s="30" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n"/>
@@ -3285,8 +3077,7 @@
       <c r="G193" s="3" t="n"/>
       <c r="H193" s="3" t="n"/>
       <c r="I193" s="3" t="n"/>
-      <c r="J193" s="3" t="n"/>
-      <c r="K193" s="30" t="n"/>
+      <c r="J193" s="30" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n"/>
@@ -3298,8 +3089,7 @@
       <c r="G194" s="3" t="n"/>
       <c r="H194" s="3" t="n"/>
       <c r="I194" s="3" t="n"/>
-      <c r="J194" s="3" t="n"/>
-      <c r="K194" s="30" t="n"/>
+      <c r="J194" s="30" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n"/>
@@ -3311,8 +3101,7 @@
       <c r="G195" s="3" t="n"/>
       <c r="H195" s="3" t="n"/>
       <c r="I195" s="3" t="n"/>
-      <c r="J195" s="3" t="n"/>
-      <c r="K195" s="30" t="n"/>
+      <c r="J195" s="30" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n"/>
@@ -3324,8 +3113,7 @@
       <c r="G196" s="3" t="n"/>
       <c r="H196" s="3" t="n"/>
       <c r="I196" s="3" t="n"/>
-      <c r="J196" s="3" t="n"/>
-      <c r="K196" s="30" t="n"/>
+      <c r="J196" s="30" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n"/>
@@ -3337,8 +3125,7 @@
       <c r="G197" s="3" t="n"/>
       <c r="H197" s="3" t="n"/>
       <c r="I197" s="3" t="n"/>
-      <c r="J197" s="3" t="n"/>
-      <c r="K197" s="30" t="n"/>
+      <c r="J197" s="30" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n"/>
@@ -3350,8 +3137,7 @@
       <c r="G198" s="3" t="n"/>
       <c r="H198" s="3" t="n"/>
       <c r="I198" s="3" t="n"/>
-      <c r="J198" s="3" t="n"/>
-      <c r="K198" s="30" t="n"/>
+      <c r="J198" s="30" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n"/>
@@ -3363,8 +3149,7 @@
       <c r="G199" s="3" t="n"/>
       <c r="H199" s="3" t="n"/>
       <c r="I199" s="3" t="n"/>
-      <c r="J199" s="3" t="n"/>
-      <c r="K199" s="30" t="n"/>
+      <c r="J199" s="30" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n"/>
@@ -3376,15 +3161,14 @@
       <c r="G200" s="3" t="n"/>
       <c r="H200" s="3" t="n"/>
       <c r="I200" s="3" t="n"/>
-      <c r="J200" s="3" t="n"/>
-      <c r="K200" s="30" t="n"/>
+      <c r="J200" s="30" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B2:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Categoría inválida" error="Usa: accesorios, ropa, zapatillas o disfraces" type="list">
+    <dataValidation sqref="B2:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"accesorios,ropa,zapatillas,tematicas"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Novedad" prompt="Pon 'sí' si es mercadería recién llegada (sale en ✨ Novedades)." type="list">
+    <dataValidation sqref="J2:J200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Novedad" prompt="Pon 'sí' si es mercadería recién llegada (sale en Novedades)." type="list">
       <formula1>"sí,no"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3713,21 +3497,21 @@
     <row r="6">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Fotos: nombres de archivo separados por coma. Ej: boina.jpg, boina-2.jpg, boina-3.jpg</t>
+          <t xml:space="preserve">   • Fotos: NO se escriben aquí. Se arrastran a la carpeta de cada producto (Irvin te la prepara).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">     👉 La PRIMERA foto es la portada. Las demás se ven al abrir el producto.</t>
+          <t xml:space="preserve">     👉 La primera foto (orden alfabético) es la portada; las demás se ven al abrir el producto.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">     👉 Sube todas esas fotos a la carpeta assets/img/productos/ del proyecto.</t>
+          <t xml:space="preserve">     👉 Se optimizan solas: no tienes que achicarlas ni renombrarlas, solo soltarlas en la carpeta.</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3573,7 @@
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>💡 Optimiza las fotos a ~100-200 KB (ancho ~800px, WebP) para que la web cargue rápido.</t>
+          <t>💡 Las fotos se optimizan automáticamente a WebP; solo arrástralas a la carpeta del producto.</t>
         </is>
       </c>
     </row>

</xml_diff>